<commit_message>
v2.7.0: HTML export now matches localhost - promo analysis, overlays, modal, promo uplift FC
</commit_message>
<xml_diff>
--- a/inputs_forecasting.xlsx
+++ b/inputs_forecasting.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fnachbar\forecasting_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA8A69A-BB91-4068-B9E1-15AFFC4D876C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0AF524-0874-4B95-A87B-B8D10E3CF522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10140" yWindow="32280" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10140" yWindow="32280" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Actuals" sheetId="1" r:id="rId1"/>
@@ -782,6 +782,1212 @@
   <dxfs count="654">
     <dxf>
       <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -920,294 +2126,6 @@
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -4735,294 +5653,6 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
@@ -6431,348 +7061,6 @@
         <shadow val="0"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
         <color rgb="FF212121"/>
         <name val="Amazon Ember"/>
         <family val="2"/>
@@ -7897,294 +8185,6 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -20827,7 +20827,7 @@
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Wk 3 2026" dataDxfId="617"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Wk 4 2026" dataDxfId="616"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Wk 5 2026" dataDxfId="615"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Wk 6 2026" dataDxfId="3"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Wk 6 2026" dataDxfId="39"/>
     <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="Wk 7 2026" dataDxfId="614"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="Wk 8 2026" dataDxfId="613"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="Wk 9 2026" dataDxfId="612"/>
@@ -20927,7 +20927,7 @@
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0100-000026000000}" name="Wk 3 2026" dataDxfId="546"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0100-000027000000}" name="Wk 4 2026" dataDxfId="545"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0100-000028000000}" name="Wk 5 2026" dataDxfId="544"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0100-000029000000}" name="Wk 6 2026" dataDxfId="0"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0100-000029000000}" name="Wk 6 2026" dataDxfId="36"/>
     <tableColumn id="42" xr3:uid="{00000000-0010-0000-0100-00002A000000}" name="Wk 7 2026" dataDxfId="543"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0100-00002B000000}" name="Wk 8 2026" dataDxfId="542"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0100-00002C000000}" name="Wk 9 2026" dataDxfId="541"/>
@@ -21023,7 +21023,7 @@
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0200-000026000000}" name="Wk 3 2026" dataDxfId="476"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0200-000027000000}" name="Wk 4 2026" dataDxfId="475"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0200-000028000000}" name="Wk 5 2026" dataDxfId="474"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0200-000029000000}" name="Wk 6 2026" dataDxfId="2"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0200-000029000000}" name="Wk 6 2026" dataDxfId="38"/>
     <tableColumn id="42" xr3:uid="{00000000-0010-0000-0200-00002A000000}" name="Wk 7 2026" dataDxfId="473"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0200-00002B000000}" name="Wk 8 2026" dataDxfId="472"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0200-00002C000000}" name="Wk 9 2026" dataDxfId="471"/>
@@ -21119,7 +21119,7 @@
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0300-000026000000}" name="Wk 3 2026" dataDxfId="388" dataCellStyle="Percent"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0300-000027000000}" name="Wk 4 2026" dataDxfId="387" dataCellStyle="Percent"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0300-000028000000}" name="Wk 5 2026" dataDxfId="386" dataCellStyle="Percent"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0300-000029000000}" name="Wk 6 2026" dataDxfId="1" dataCellStyle="Percent"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0300-000029000000}" name="Wk 6 2026" dataDxfId="37" dataCellStyle="Percent"/>
     <tableColumn id="42" xr3:uid="{00000000-0010-0000-0300-00002A000000}" name="Wk 7 2026" dataDxfId="385" dataCellStyle="Percent"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0300-00002B000000}" name="Wk 8 2026" dataDxfId="384" dataCellStyle="Percent"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0300-00002C000000}" name="Wk 9 2026" dataDxfId="383" dataCellStyle="Percent"/>
@@ -21240,264 +21240,262 @@
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0400-00002C000000}" name="Wk 9 2026" dataDxfId="297">
       <calculatedColumnFormula>AS15*AS26*AS37</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0400-00002D000000}" name="Wk 10 2026" dataDxfId="296">
-      <calculatedColumnFormula>AT15*AT26*AT37</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0400-00002E000000}" name="Wk 11 2026" dataDxfId="295"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0400-00002F000000}" name="Wk 12 2026" dataDxfId="294"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0400-000030000000}" name="Wk 13 2026" dataDxfId="293"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0400-000031000000}" name="Wk 14 2026" dataDxfId="292"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0400-000032000000}" name="Wk 15 2026" dataDxfId="291"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0400-000033000000}" name="Wk 16 2026" dataDxfId="290"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0400-000034000000}" name="Wk 17 2026" dataDxfId="289"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0400-000035000000}" name="Wk 18 2026" dataDxfId="288"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0400-000036000000}" name="Wk 19 2026" dataDxfId="287"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0400-000037000000}" name="Wk 20 2026" dataDxfId="286"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0400-000038000000}" name="Wk 21 2026" dataDxfId="285"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0400-000039000000}" name="Wk 22 2026" dataDxfId="284"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0400-00003A000000}" name="Wk 23 2026" dataDxfId="283"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0400-00003B000000}" name="Wk 24 2026" dataDxfId="282"/>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0400-00003C000000}" name="Wk 25 2026" dataDxfId="281"/>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0400-00003D000000}" name="Wk 26 2026" dataDxfId="280"/>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0400-00003E000000}" name="Wk 27 2026" dataDxfId="279"/>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0400-00003F000000}" name="Wk 28 2026" dataDxfId="278"/>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0400-000040000000}" name="Wk 29 2026" dataDxfId="277"/>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0400-000041000000}" name="Wk 30 2026" dataDxfId="276"/>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0400-000042000000}" name="Wk 31 2026" dataDxfId="275"/>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0400-000043000000}" name="Wk 32 2026" dataDxfId="274"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0400-000044000000}" name="Wk 33 2026" dataDxfId="273"/>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0400-000045000000}" name="Wk 34 2026" dataDxfId="272"/>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0400-000046000000}" name="Wk 35 2026" dataDxfId="271"/>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0400-000047000000}" name="Wk 36 2026" dataDxfId="270"/>
-    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0400-000048000000}" name="Wk 37 2026" dataDxfId="269"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0400-000049000000}" name="Wk 38 2026" dataDxfId="268"/>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0400-00004A000000}" name="Wk 39 2026" dataDxfId="267"/>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0400-00004B000000}" name="Wk 40 2026" dataDxfId="266"/>
-    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0400-00004C000000}" name="Wk 41 2026" dataDxfId="265"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0400-00004D000000}" name="Wk 42 2026" dataDxfId="264"/>
-    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0400-00004E000000}" name="Wk 43 2026" dataDxfId="263"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0400-00004F000000}" name="Wk 44 2026" dataDxfId="262"/>
-    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0400-000050000000}" name="Wk 45 2026" dataDxfId="261"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0400-000051000000}" name="Wk 46 2026" dataDxfId="260"/>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0400-000052000000}" name="Wk 47 2026" dataDxfId="259"/>
-    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0400-000053000000}" name="Wk 48 2026" dataDxfId="258"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0400-000054000000}" name="Wk 49 2026" dataDxfId="257"/>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0400-000055000000}" name="Wk 50 2026" dataDxfId="256"/>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0400-000056000000}" name="Wk 51 2026" dataDxfId="255"/>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0400-000057000000}" name="Wk 52 2026" dataDxfId="254"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0400-00002D000000}" name="Wk 10 2026" dataDxfId="8"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0400-00002E000000}" name="Wk 11 2026" dataDxfId="7"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0400-00002F000000}" name="Wk 12 2026" dataDxfId="6"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0400-000030000000}" name="Wk 13 2026" dataDxfId="5"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0400-000031000000}" name="Wk 14 2026" dataDxfId="4"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0400-000032000000}" name="Wk 15 2026" dataDxfId="3"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0400-000033000000}" name="Wk 16 2026" dataDxfId="2"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0400-000034000000}" name="Wk 17 2026" dataDxfId="1"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0400-000035000000}" name="Wk 18 2026" dataDxfId="0"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0400-000036000000}" name="Wk 19 2026" dataDxfId="296"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0400-000037000000}" name="Wk 20 2026" dataDxfId="295"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0400-000038000000}" name="Wk 21 2026" dataDxfId="294"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0400-000039000000}" name="Wk 22 2026" dataDxfId="293"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0400-00003A000000}" name="Wk 23 2026" dataDxfId="292"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0400-00003B000000}" name="Wk 24 2026" dataDxfId="291"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0400-00003C000000}" name="Wk 25 2026" dataDxfId="290"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0400-00003D000000}" name="Wk 26 2026" dataDxfId="289"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0400-00003E000000}" name="Wk 27 2026" dataDxfId="288"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0400-00003F000000}" name="Wk 28 2026" dataDxfId="287"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0400-000040000000}" name="Wk 29 2026" dataDxfId="286"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0400-000041000000}" name="Wk 30 2026" dataDxfId="285"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0400-000042000000}" name="Wk 31 2026" dataDxfId="284"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0400-000043000000}" name="Wk 32 2026" dataDxfId="283"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0400-000044000000}" name="Wk 33 2026" dataDxfId="282"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0400-000045000000}" name="Wk 34 2026" dataDxfId="281"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0400-000046000000}" name="Wk 35 2026" dataDxfId="280"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0400-000047000000}" name="Wk 36 2026" dataDxfId="279"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0400-000048000000}" name="Wk 37 2026" dataDxfId="278"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0400-000049000000}" name="Wk 38 2026" dataDxfId="277"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0400-00004A000000}" name="Wk 39 2026" dataDxfId="276"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0400-00004B000000}" name="Wk 40 2026" dataDxfId="275"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0400-00004C000000}" name="Wk 41 2026" dataDxfId="274"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0400-00004D000000}" name="Wk 42 2026" dataDxfId="273"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0400-00004E000000}" name="Wk 43 2026" dataDxfId="272"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0400-00004F000000}" name="Wk 44 2026" dataDxfId="271"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0400-000050000000}" name="Wk 45 2026" dataDxfId="270"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0400-000051000000}" name="Wk 46 2026" dataDxfId="269"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0400-000052000000}" name="Wk 47 2026" dataDxfId="268"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0400-000053000000}" name="Wk 48 2026" dataDxfId="267"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0400-000054000000}" name="Wk 49 2026" dataDxfId="266"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0400-000055000000}" name="Wk 50 2026" dataDxfId="265"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0400-000056000000}" name="Wk 51 2026" dataDxfId="264"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0400-000057000000}" name="Wk 52 2026" dataDxfId="263"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblForecastTransits25" displayName="tblForecastTransits25" ref="B14:CJ20" totalsRowShown="0" headerRowDxfId="253" dataDxfId="251" headerRowBorderDxfId="252" tableBorderDxfId="250">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblForecastTransits25" displayName="tblForecastTransits25" ref="B14:CJ20" totalsRowShown="0" headerRowDxfId="262" dataDxfId="260" headerRowBorderDxfId="261" tableBorderDxfId="259">
   <autoFilter ref="B14:CJ20" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="87">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="MP"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Wk19 2025" dataDxfId="249"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Wk20 2025" dataDxfId="248"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Wk21 2025" dataDxfId="247"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Wk22 2025" dataDxfId="246"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wk23 2025" dataDxfId="245"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="Wk24 2025" dataDxfId="244"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Wk25 2025" dataDxfId="243"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="Wk26 2025" dataDxfId="242"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="Wk27 2025" dataDxfId="241"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="Wk28 2025" dataDxfId="240"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="Wk29 2025" dataDxfId="239"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0500-00000D000000}" name="Wk30 2025" dataDxfId="238"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0500-00000E000000}" name="Wk31 2025" dataDxfId="237"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="Wk32 2025" dataDxfId="236"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0500-000010000000}" name="Wk33 2025" dataDxfId="235"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0500-000011000000}" name="Wk34 2025" dataDxfId="234"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0500-000012000000}" name="Wk35 2025" dataDxfId="233"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0500-000013000000}" name="Wk36 2025" dataDxfId="232"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0500-000014000000}" name="Wk37 2025" dataDxfId="231"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0500-000015000000}" name="Wk38 2025" dataDxfId="230"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0500-000016000000}" name="Wk39 2025" dataDxfId="229"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0500-000017000000}" name="Wk40 2025" dataDxfId="228"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0500-000018000000}" name="Wk41 2025" dataDxfId="227"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0500-000019000000}" name="Wk42 2025" dataDxfId="226"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0500-00001A000000}" name="Wk43 2025" dataDxfId="225"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0500-00001B000000}" name="Wk44 2025" dataDxfId="224"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0500-00001C000000}" name="Wk45 2025" dataDxfId="223"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0500-00001D000000}" name="Wk46 2025" dataDxfId="222"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0500-00001E000000}" name="Wk47 2025" dataDxfId="221"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0500-00001F000000}" name="Wk48 2025" dataDxfId="220"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0500-000020000000}" name="Wk49 2025" dataDxfId="219"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0500-000021000000}" name="Wk50 2025" dataDxfId="218"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0500-000022000000}" name="Wk51 2025" dataDxfId="217"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0500-000023000000}" name="Wk52 2025" dataDxfId="216"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0500-000024000000}" name="Wk 1 2026" dataDxfId="215"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0500-000025000000}" name="Wk 2 2026" dataDxfId="214"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0500-000026000000}" name="Wk 3 2026" dataDxfId="213"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0500-000027000000}" name="Wk 4 2026" dataDxfId="212"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0500-000028000000}" name="Wk 5 2026" dataDxfId="211"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0500-000029000000}" name="Wk 6 2026" dataDxfId="210"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0500-00002A000000}" name="Wk 7 2026" dataDxfId="209"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0500-00002B000000}" name="Wk 8 2026" dataDxfId="208"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0500-00002C000000}" name="Wk 9 2026" dataDxfId="207"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0500-00002D000000}" name="Wk 10 2026" dataDxfId="206"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0500-00002E000000}" name="Wk 11 2026" dataDxfId="205"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0500-00002F000000}" name="Wk 12 2026" dataDxfId="204"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0500-000030000000}" name="Wk 13 2026" dataDxfId="203"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0500-000031000000}" name="Wk 14 2026" dataDxfId="202"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0500-000032000000}" name="Wk 15 2026" dataDxfId="201"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0500-000033000000}" name="Wk 16 2026" dataDxfId="200"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0500-000034000000}" name="Wk 17 2026" dataDxfId="199"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0500-000035000000}" name="Wk 18 2026" dataDxfId="198"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0500-000036000000}" name="Wk 19 2026" dataDxfId="197"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0500-000037000000}" name="Wk 20 2026" dataDxfId="196"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0500-000038000000}" name="Wk 21 2026" dataDxfId="195"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0500-000039000000}" name="Wk 22 2026" dataDxfId="194"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0500-00003A000000}" name="Wk 23 2026" dataDxfId="193"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0500-00003B000000}" name="Wk 24 2026" dataDxfId="192"/>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0500-00003C000000}" name="Wk 25 2026" dataDxfId="191"/>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0500-00003D000000}" name="Wk 26 2026" dataDxfId="190"/>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0500-00003E000000}" name="Wk 27 2026" dataDxfId="189"/>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0500-00003F000000}" name="Wk 28 2026" dataDxfId="188"/>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0500-000040000000}" name="Wk 29 2026" dataDxfId="187"/>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0500-000041000000}" name="Wk 30 2026" dataDxfId="186"/>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0500-000042000000}" name="Wk 31 2026" dataDxfId="185"/>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0500-000043000000}" name="Wk 32 2026" dataDxfId="184"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0500-000044000000}" name="Wk 33 2026" dataDxfId="183"/>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0500-000045000000}" name="Wk 34 2026" dataDxfId="182"/>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0500-000046000000}" name="Wk 35 2026" dataDxfId="181"/>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0500-000047000000}" name="Wk 36 2026" dataDxfId="180"/>
-    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0500-000048000000}" name="Wk 37 2026" dataDxfId="179"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0500-000049000000}" name="Wk 38 2026" dataDxfId="178"/>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0500-00004A000000}" name="Wk 39 2026" dataDxfId="177"/>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0500-00004B000000}" name="Wk 40 2026" dataDxfId="176"/>
-    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0500-00004C000000}" name="Wk 41 2026" dataDxfId="175"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0500-00004D000000}" name="Wk 42 2026" dataDxfId="174"/>
-    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0500-00004E000000}" name="Wk 43 2026" dataDxfId="173"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0500-00004F000000}" name="Wk 44 2026" dataDxfId="172"/>
-    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0500-000050000000}" name="Wk 45 2026" dataDxfId="171"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0500-000051000000}" name="Wk 46 2026" dataDxfId="170"/>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0500-000052000000}" name="Wk 47 2026" dataDxfId="169"/>
-    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0500-000053000000}" name="Wk 48 2026" dataDxfId="168"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0500-000054000000}" name="Wk 49 2026" dataDxfId="167"/>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0500-000055000000}" name="Wk 50 2026" dataDxfId="166"/>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0500-000056000000}" name="Wk 51 2026" dataDxfId="165"/>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0500-000057000000}" name="Wk 52 2026" dataDxfId="164"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Wk19 2025" dataDxfId="258"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Wk20 2025" dataDxfId="257"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Wk21 2025" dataDxfId="256"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Wk22 2025" dataDxfId="255"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wk23 2025" dataDxfId="254"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="Wk24 2025" dataDxfId="253"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Wk25 2025" dataDxfId="252"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="Wk26 2025" dataDxfId="251"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="Wk27 2025" dataDxfId="250"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="Wk28 2025" dataDxfId="249"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="Wk29 2025" dataDxfId="248"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0500-00000D000000}" name="Wk30 2025" dataDxfId="247"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0500-00000E000000}" name="Wk31 2025" dataDxfId="246"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="Wk32 2025" dataDxfId="245"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0500-000010000000}" name="Wk33 2025" dataDxfId="244"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0500-000011000000}" name="Wk34 2025" dataDxfId="243"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0500-000012000000}" name="Wk35 2025" dataDxfId="242"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0500-000013000000}" name="Wk36 2025" dataDxfId="241"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0500-000014000000}" name="Wk37 2025" dataDxfId="240"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0500-000015000000}" name="Wk38 2025" dataDxfId="239"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0500-000016000000}" name="Wk39 2025" dataDxfId="238"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0500-000017000000}" name="Wk40 2025" dataDxfId="237"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0500-000018000000}" name="Wk41 2025" dataDxfId="236"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0500-000019000000}" name="Wk42 2025" dataDxfId="235"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0500-00001A000000}" name="Wk43 2025" dataDxfId="234"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0500-00001B000000}" name="Wk44 2025" dataDxfId="233"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0500-00001C000000}" name="Wk45 2025" dataDxfId="232"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0500-00001D000000}" name="Wk46 2025" dataDxfId="231"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0500-00001E000000}" name="Wk47 2025" dataDxfId="230"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0500-00001F000000}" name="Wk48 2025" dataDxfId="229"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0500-000020000000}" name="Wk49 2025" dataDxfId="228"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0500-000021000000}" name="Wk50 2025" dataDxfId="227"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0500-000022000000}" name="Wk51 2025" dataDxfId="226"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0500-000023000000}" name="Wk52 2025" dataDxfId="225"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0500-000024000000}" name="Wk 1 2026" dataDxfId="224"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0500-000025000000}" name="Wk 2 2026" dataDxfId="223"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0500-000026000000}" name="Wk 3 2026" dataDxfId="222"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0500-000027000000}" name="Wk 4 2026" dataDxfId="221"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0500-000028000000}" name="Wk 5 2026" dataDxfId="220"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0500-000029000000}" name="Wk 6 2026" dataDxfId="219"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0500-00002A000000}" name="Wk 7 2026" dataDxfId="218"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0500-00002B000000}" name="Wk 8 2026" dataDxfId="217"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0500-00002C000000}" name="Wk 9 2026" dataDxfId="216"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0500-00002D000000}" name="Wk 10 2026" dataDxfId="35"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0500-00002E000000}" name="Wk 11 2026" dataDxfId="34"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0500-00002F000000}" name="Wk 12 2026" dataDxfId="33"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0500-000030000000}" name="Wk 13 2026" dataDxfId="32"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0500-000031000000}" name="Wk 14 2026" dataDxfId="31"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0500-000032000000}" name="Wk 15 2026" dataDxfId="30"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0500-000033000000}" name="Wk 16 2026" dataDxfId="29"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0500-000034000000}" name="Wk 17 2026" dataDxfId="28"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0500-000035000000}" name="Wk 18 2026" dataDxfId="27"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0500-000036000000}" name="Wk 19 2026" dataDxfId="215"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0500-000037000000}" name="Wk 20 2026" dataDxfId="214"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0500-000038000000}" name="Wk 21 2026" dataDxfId="213"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0500-000039000000}" name="Wk 22 2026" dataDxfId="212"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0500-00003A000000}" name="Wk 23 2026" dataDxfId="211"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0500-00003B000000}" name="Wk 24 2026" dataDxfId="210"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0500-00003C000000}" name="Wk 25 2026" dataDxfId="209"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0500-00003D000000}" name="Wk 26 2026" dataDxfId="208"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0500-00003E000000}" name="Wk 27 2026" dataDxfId="207"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0500-00003F000000}" name="Wk 28 2026" dataDxfId="206"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0500-000040000000}" name="Wk 29 2026" dataDxfId="205"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0500-000041000000}" name="Wk 30 2026" dataDxfId="204"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0500-000042000000}" name="Wk 31 2026" dataDxfId="203"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0500-000043000000}" name="Wk 32 2026" dataDxfId="202"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0500-000044000000}" name="Wk 33 2026" dataDxfId="201"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0500-000045000000}" name="Wk 34 2026" dataDxfId="200"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0500-000046000000}" name="Wk 35 2026" dataDxfId="199"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0500-000047000000}" name="Wk 36 2026" dataDxfId="198"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0500-000048000000}" name="Wk 37 2026" dataDxfId="197"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0500-000049000000}" name="Wk 38 2026" dataDxfId="196"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0500-00004A000000}" name="Wk 39 2026" dataDxfId="195"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0500-00004B000000}" name="Wk 40 2026" dataDxfId="194"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0500-00004C000000}" name="Wk 41 2026" dataDxfId="193"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0500-00004D000000}" name="Wk 42 2026" dataDxfId="192"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0500-00004E000000}" name="Wk 43 2026" dataDxfId="191"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0500-00004F000000}" name="Wk 44 2026" dataDxfId="190"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0500-000050000000}" name="Wk 45 2026" dataDxfId="189"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0500-000051000000}" name="Wk 46 2026" dataDxfId="188"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0500-000052000000}" name="Wk 47 2026" dataDxfId="187"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0500-000053000000}" name="Wk 48 2026" dataDxfId="186"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0500-000054000000}" name="Wk 49 2026" dataDxfId="185"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0500-000055000000}" name="Wk 50 2026" dataDxfId="184"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0500-000056000000}" name="Wk 51 2026" dataDxfId="183"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0500-000057000000}" name="Wk 52 2026" dataDxfId="182"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblForecastConversion26" displayName="tblForecastConversion26" ref="B25:CJ31" totalsRowShown="0" headerRowDxfId="163" headerRowBorderDxfId="162" tableBorderDxfId="161">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblForecastConversion26" displayName="tblForecastConversion26" ref="B25:CJ31" totalsRowShown="0" headerRowDxfId="181" headerRowBorderDxfId="180" tableBorderDxfId="179">
   <autoFilter ref="B25:CJ31" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="87">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="MP"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Wk19 2025" dataDxfId="160"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Wk20 2025" dataDxfId="159"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Wk21 2025" dataDxfId="158"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Wk22 2025" dataDxfId="157"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Wk23 2025" dataDxfId="156"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="Wk24 2025" dataDxfId="155"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="Wk25 2025" dataDxfId="154"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="Wk26 2025" dataDxfId="153"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" name="Wk27 2025" dataDxfId="152"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" name="Wk28 2025" dataDxfId="151"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" name="Wk29 2025" dataDxfId="150"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" name="Wk30 2025" dataDxfId="149"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" name="Wk31 2025" dataDxfId="148"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" name="Wk32 2025" dataDxfId="147"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" name="Wk33 2025" dataDxfId="146"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" name="Wk34 2025" dataDxfId="145"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0600-000012000000}" name="Wk35 2025" dataDxfId="144"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0600-000013000000}" name="Wk36 2025" dataDxfId="143"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0600-000014000000}" name="Wk37 2025" dataDxfId="142"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0600-000015000000}" name="Wk38 2025" dataDxfId="141"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0600-000016000000}" name="Wk39 2025" dataDxfId="140"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0600-000017000000}" name="Wk40 2025" dataDxfId="139"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0600-000018000000}" name="Wk41 2025" dataDxfId="138"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0600-000019000000}" name="Wk42 2025" dataDxfId="137"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0600-00001A000000}" name="Wk43 2025" dataDxfId="136"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0600-00001B000000}" name="Wk44 2025" dataDxfId="135"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0600-00001C000000}" name="Wk45 2025" dataDxfId="134"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0600-00001D000000}" name="Wk46 2025" dataDxfId="133"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0600-00001E000000}" name="Wk47 2025" dataDxfId="132"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0600-00001F000000}" name="Wk48 2025" dataDxfId="131"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0600-000020000000}" name="Wk49 2025" dataDxfId="130"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0600-000021000000}" name="Wk50 2025" dataDxfId="129"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0600-000022000000}" name="Wk51 2025" dataDxfId="128"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0600-000023000000}" name="Wk52 2025" dataDxfId="127"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0600-000024000000}" name="Wk 1 2026" dataDxfId="126"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0600-000025000000}" name="Wk 2 2026" dataDxfId="125"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0600-000026000000}" name="Wk 3 2026" dataDxfId="124"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0600-000027000000}" name="Wk 4 2026" dataDxfId="123"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0600-000028000000}" name="Wk 5 2026" dataDxfId="122"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0600-000029000000}" name="Wk 6 2026" dataDxfId="121"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0600-00002A000000}" name="Wk 7 2026" dataDxfId="120"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0600-00002B000000}" name="Wk 8 2026" dataDxfId="119"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0600-00002C000000}" name="Wk 9 2026" dataDxfId="118"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0600-00002D000000}" name="Wk 10 2026" dataDxfId="117"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0600-00002E000000}" name="Wk 11 2026" dataDxfId="116"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0600-00002F000000}" name="Wk 12 2026" dataDxfId="115"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0600-000030000000}" name="Wk 13 2026" dataDxfId="114"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0600-000031000000}" name="Wk 14 2026" dataDxfId="113"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0600-000032000000}" name="Wk 15 2026" dataDxfId="112"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0600-000033000000}" name="Wk 16 2026" dataDxfId="111"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0600-000034000000}" name="Wk 17 2026" dataDxfId="110"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0600-000035000000}" name="Wk 18 2026" dataDxfId="109"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0600-000036000000}" name="Wk 19 2026" dataDxfId="108"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0600-000037000000}" name="Wk 20 2026" dataDxfId="107"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0600-000038000000}" name="Wk 21 2026" dataDxfId="106"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0600-000039000000}" name="Wk 22 2026" dataDxfId="105"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0600-00003A000000}" name="Wk 23 2026" dataDxfId="104"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0600-00003B000000}" name="Wk 24 2026" dataDxfId="103"/>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0600-00003C000000}" name="Wk 25 2026" dataDxfId="102"/>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0600-00003D000000}" name="Wk 26 2026" dataDxfId="101"/>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0600-00003E000000}" name="Wk 27 2026" dataDxfId="100"/>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0600-00003F000000}" name="Wk 28 2026" dataDxfId="99"/>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0600-000040000000}" name="Wk 29 2026" dataDxfId="98"/>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0600-000041000000}" name="Wk 30 2026" dataDxfId="97"/>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0600-000042000000}" name="Wk 31 2026" dataDxfId="96"/>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0600-000043000000}" name="Wk 32 2026" dataDxfId="95"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0600-000044000000}" name="Wk 33 2026" dataDxfId="94"/>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0600-000045000000}" name="Wk 34 2026" dataDxfId="93"/>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0600-000046000000}" name="Wk 35 2026" dataDxfId="92"/>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0600-000047000000}" name="Wk 36 2026" dataDxfId="91"/>
-    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0600-000048000000}" name="Wk 37 2026" dataDxfId="90"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0600-000049000000}" name="Wk 38 2026" dataDxfId="89"/>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0600-00004A000000}" name="Wk 39 2026" dataDxfId="88"/>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0600-00004B000000}" name="Wk 40 2026" dataDxfId="87"/>
-    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0600-00004C000000}" name="Wk 41 2026" dataDxfId="86"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0600-00004D000000}" name="Wk 42 2026" dataDxfId="85"/>
-    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0600-00004E000000}" name="Wk 43 2026" dataDxfId="84"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0600-00004F000000}" name="Wk 44 2026" dataDxfId="83"/>
-    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0600-000050000000}" name="Wk 45 2026" dataDxfId="82"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0600-000051000000}" name="Wk 46 2026" dataDxfId="81"/>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0600-000052000000}" name="Wk 47 2026" dataDxfId="80"/>
-    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0600-000053000000}" name="Wk 48 2026" dataDxfId="79"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0600-000054000000}" name="Wk 49 2026" dataDxfId="78"/>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0600-000055000000}" name="Wk 50 2026" dataDxfId="77"/>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0600-000056000000}" name="Wk 51 2026" dataDxfId="76"/>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0600-000057000000}" name="Wk 52 2026" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Wk19 2025" dataDxfId="178"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Wk20 2025" dataDxfId="177"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Wk21 2025" dataDxfId="176"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Wk22 2025" dataDxfId="175"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Wk23 2025" dataDxfId="174"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="Wk24 2025" dataDxfId="173"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="Wk25 2025" dataDxfId="172"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="Wk26 2025" dataDxfId="171"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" name="Wk27 2025" dataDxfId="170"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" name="Wk28 2025" dataDxfId="169"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" name="Wk29 2025" dataDxfId="168"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" name="Wk30 2025" dataDxfId="167"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" name="Wk31 2025" dataDxfId="166"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" name="Wk32 2025" dataDxfId="165"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" name="Wk33 2025" dataDxfId="164"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" name="Wk34 2025" dataDxfId="163"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0600-000012000000}" name="Wk35 2025" dataDxfId="162"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0600-000013000000}" name="Wk36 2025" dataDxfId="161"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0600-000014000000}" name="Wk37 2025" dataDxfId="160"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0600-000015000000}" name="Wk38 2025" dataDxfId="159"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0600-000016000000}" name="Wk39 2025" dataDxfId="158"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0600-000017000000}" name="Wk40 2025" dataDxfId="157"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0600-000018000000}" name="Wk41 2025" dataDxfId="156"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0600-000019000000}" name="Wk42 2025" dataDxfId="155"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0600-00001A000000}" name="Wk43 2025" dataDxfId="154"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0600-00001B000000}" name="Wk44 2025" dataDxfId="153"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0600-00001C000000}" name="Wk45 2025" dataDxfId="152"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0600-00001D000000}" name="Wk46 2025" dataDxfId="151"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0600-00001E000000}" name="Wk47 2025" dataDxfId="150"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0600-00001F000000}" name="Wk48 2025" dataDxfId="149"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0600-000020000000}" name="Wk49 2025" dataDxfId="148"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0600-000021000000}" name="Wk50 2025" dataDxfId="147"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0600-000022000000}" name="Wk51 2025" dataDxfId="146"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0600-000023000000}" name="Wk52 2025" dataDxfId="145"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0600-000024000000}" name="Wk 1 2026" dataDxfId="144"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0600-000025000000}" name="Wk 2 2026" dataDxfId="143"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0600-000026000000}" name="Wk 3 2026" dataDxfId="142"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0600-000027000000}" name="Wk 4 2026" dataDxfId="141"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0600-000028000000}" name="Wk 5 2026" dataDxfId="140"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0600-000029000000}" name="Wk 6 2026" dataDxfId="139"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0600-00002A000000}" name="Wk 7 2026" dataDxfId="138"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0600-00002B000000}" name="Wk 8 2026" dataDxfId="137"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0600-00002C000000}" name="Wk 9 2026" dataDxfId="136"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0600-00002D000000}" name="Wk 10 2026" dataDxfId="26"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0600-00002E000000}" name="Wk 11 2026" dataDxfId="25"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0600-00002F000000}" name="Wk 12 2026" dataDxfId="24"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0600-000030000000}" name="Wk 13 2026" dataDxfId="23"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0600-000031000000}" name="Wk 14 2026" dataDxfId="22"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0600-000032000000}" name="Wk 15 2026" dataDxfId="21"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0600-000033000000}" name="Wk 16 2026" dataDxfId="20"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0600-000034000000}" name="Wk 17 2026" dataDxfId="19"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0600-000035000000}" name="Wk 18 2026" dataDxfId="18"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0600-000036000000}" name="Wk 19 2026" dataDxfId="135"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0600-000037000000}" name="Wk 20 2026" dataDxfId="134"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0600-000038000000}" name="Wk 21 2026" dataDxfId="133"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0600-000039000000}" name="Wk 22 2026" dataDxfId="132"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0600-00003A000000}" name="Wk 23 2026" dataDxfId="131"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0600-00003B000000}" name="Wk 24 2026" dataDxfId="130"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0600-00003C000000}" name="Wk 25 2026" dataDxfId="129"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0600-00003D000000}" name="Wk 26 2026" dataDxfId="128"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0600-00003E000000}" name="Wk 27 2026" dataDxfId="127"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0600-00003F000000}" name="Wk 28 2026" dataDxfId="126"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0600-000040000000}" name="Wk 29 2026" dataDxfId="125"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0600-000041000000}" name="Wk 30 2026" dataDxfId="124"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0600-000042000000}" name="Wk 31 2026" dataDxfId="123"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0600-000043000000}" name="Wk 32 2026" dataDxfId="122"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0600-000044000000}" name="Wk 33 2026" dataDxfId="121"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0600-000045000000}" name="Wk 34 2026" dataDxfId="120"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0600-000046000000}" name="Wk 35 2026" dataDxfId="119"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0600-000047000000}" name="Wk 36 2026" dataDxfId="118"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0600-000048000000}" name="Wk 37 2026" dataDxfId="117"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0600-000049000000}" name="Wk 38 2026" dataDxfId="116"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0600-00004A000000}" name="Wk 39 2026" dataDxfId="115"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0600-00004B000000}" name="Wk 40 2026" dataDxfId="114"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0600-00004C000000}" name="Wk 41 2026" dataDxfId="113"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0600-00004D000000}" name="Wk 42 2026" dataDxfId="112"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0600-00004E000000}" name="Wk 43 2026" dataDxfId="111"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0600-00004F000000}" name="Wk 44 2026" dataDxfId="110"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0600-000050000000}" name="Wk 45 2026" dataDxfId="109"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0600-000051000000}" name="Wk 46 2026" dataDxfId="108"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0600-000052000000}" name="Wk 47 2026" dataDxfId="107"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0600-000053000000}" name="Wk 48 2026" dataDxfId="106"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0600-000054000000}" name="Wk 49 2026" dataDxfId="105"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0600-000055000000}" name="Wk 50 2026" dataDxfId="104"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0600-000056000000}" name="Wk 51 2026" dataDxfId="103"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0600-000057000000}" name="Wk 52 2026" dataDxfId="102"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="TblForecastUPO27" displayName="TblForecastUPO27" ref="B36:CJ42" totalsRowShown="0" headerRowDxfId="74" headerRowBorderDxfId="73" tableBorderDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="TblForecastUPO27" displayName="TblForecastUPO27" ref="B36:CJ42" totalsRowShown="0" headerRowDxfId="101" headerRowBorderDxfId="100" tableBorderDxfId="99">
   <autoFilter ref="B36:CJ42" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="87">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="MP"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Wk19 2025" dataDxfId="71"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Wk20 2025" dataDxfId="70"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Wk21 2025" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Wk19 2025" dataDxfId="98"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Wk20 2025" dataDxfId="97"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Wk21 2025" dataDxfId="96"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Wk22 2025"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Wk23 2025"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Wk24 2025"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Wk25 2025"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Wk26 2025"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Wk27 2025"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Wk28 2025" dataDxfId="68"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Wk29 2025" dataDxfId="67"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Wk28 2025" dataDxfId="95"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Wk29 2025" dataDxfId="94"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0700-00000D000000}" name="Wk30 2025"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0700-00000E000000}" name="Wk31 2025"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0700-00000F000000}" name="Wk32 2025"/>
@@ -21510,69 +21508,69 @@
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0700-000016000000}" name="Wk39 2025"/>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0700-000017000000}" name="Wk40 2025"/>
     <tableColumn id="24" xr3:uid="{00000000-0010-0000-0700-000018000000}" name="Wk41 2025"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0700-000019000000}" name="Wk42 2025" dataDxfId="66"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0700-00001A000000}" name="Wk43 2025" dataDxfId="65"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0700-00001B000000}" name="Wk44 2025" dataDxfId="64"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0700-00001C000000}" name="Wk45 2025" dataDxfId="63"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="Wk46 2025" dataDxfId="62"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0700-00001E000000}" name="Wk47 2025" dataDxfId="61"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0700-00001F000000}" name="Wk48 2025" dataDxfId="60"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0700-000020000000}" name="Wk49 2025" dataDxfId="59"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0700-000021000000}" name="Wk50 2025" dataDxfId="58"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0700-000022000000}" name="Wk51 2025" dataDxfId="57"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0700-000023000000}" name="Wk52 2025" dataDxfId="56"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0700-000024000000}" name="Wk 1 2026" dataDxfId="55"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0700-000025000000}" name="Wk 2 2026" dataDxfId="54"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0700-000026000000}" name="Wk 3 2026" dataDxfId="53"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0700-000027000000}" name="Wk 4 2026" dataDxfId="52"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0700-000028000000}" name="Wk 5 2026" dataDxfId="51"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0700-000029000000}" name="Wk 6 2026" dataDxfId="50"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0700-00002A000000}" name="Wk 7 2026" dataDxfId="49"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0700-00002B000000}" name="Wk 8 2026" dataDxfId="48"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0700-00002C000000}" name="Wk 9 2026" dataDxfId="47"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0700-00002D000000}" name="Wk 10 2026" dataDxfId="46"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0700-00002E000000}" name="Wk 11 2026" dataDxfId="45"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0700-00002F000000}" name="Wk 12 2026" dataDxfId="44"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0700-000030000000}" name="Wk 13 2026" dataDxfId="43"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0700-000031000000}" name="Wk 14 2026" dataDxfId="42"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0700-000032000000}" name="Wk 15 2026" dataDxfId="41"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0700-000033000000}" name="Wk 16 2026" dataDxfId="40"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0700-000034000000}" name="Wk 17 2026" dataDxfId="39"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0700-000035000000}" name="Wk 18 2026" dataDxfId="38"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0700-000036000000}" name="Wk 19 2026" dataDxfId="37"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0700-000037000000}" name="Wk 20 2026" dataDxfId="36"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0700-000038000000}" name="Wk 21 2026" dataDxfId="35"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0700-000039000000}" name="Wk 22 2026" dataDxfId="34"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0700-00003A000000}" name="Wk 23 2026" dataDxfId="33"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0700-00003B000000}" name="Wk 24 2026" dataDxfId="32"/>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0700-00003C000000}" name="Wk 25 2026" dataDxfId="31"/>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0700-00003D000000}" name="Wk 26 2026" dataDxfId="30"/>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0700-00003E000000}" name="Wk 27 2026" dataDxfId="29"/>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0700-00003F000000}" name="Wk 28 2026" dataDxfId="28"/>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0700-000040000000}" name="Wk 29 2026" dataDxfId="27"/>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0700-000041000000}" name="Wk 30 2026" dataDxfId="26"/>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0700-000042000000}" name="Wk 31 2026" dataDxfId="25"/>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0700-000043000000}" name="Wk 32 2026" dataDxfId="24"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0700-000044000000}" name="Wk 33 2026" dataDxfId="23"/>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0700-000045000000}" name="Wk 34 2026" dataDxfId="22"/>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0700-000046000000}" name="Wk 35 2026" dataDxfId="21"/>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0700-000047000000}" name="Wk 36 2026" dataDxfId="20"/>
-    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0700-000048000000}" name="Wk 37 2026" dataDxfId="19"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0700-000049000000}" name="Wk 38 2026" dataDxfId="18"/>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0700-00004A000000}" name="Wk 39 2026" dataDxfId="17"/>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0700-00004B000000}" name="Wk 40 2026" dataDxfId="16"/>
-    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0700-00004C000000}" name="Wk 41 2026" dataDxfId="15"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0700-00004D000000}" name="Wk 42 2026" dataDxfId="14"/>
-    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0700-00004E000000}" name="Wk 43 2026" dataDxfId="13"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0700-00004F000000}" name="Wk 44 2026" dataDxfId="12"/>
-    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0700-000050000000}" name="Wk 45 2026" dataDxfId="11"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0700-000051000000}" name="Wk 46 2026" dataDxfId="10"/>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0700-000052000000}" name="Wk 47 2026" dataDxfId="9"/>
-    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0700-000053000000}" name="Wk 48 2026" dataDxfId="8"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0700-000054000000}" name="Wk 49 2026" dataDxfId="7"/>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0700-000055000000}" name="Wk 50 2026" dataDxfId="6"/>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0700-000056000000}" name="Wk 51 2026" dataDxfId="5"/>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0700-000057000000}" name="Wk 52 2026" dataDxfId="4"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0700-000019000000}" name="Wk42 2025" dataDxfId="93"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0700-00001A000000}" name="Wk43 2025" dataDxfId="92"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0700-00001B000000}" name="Wk44 2025" dataDxfId="91"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0700-00001C000000}" name="Wk45 2025" dataDxfId="90"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="Wk46 2025" dataDxfId="89"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0700-00001E000000}" name="Wk47 2025" dataDxfId="88"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0700-00001F000000}" name="Wk48 2025" dataDxfId="87"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0700-000020000000}" name="Wk49 2025" dataDxfId="86"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0700-000021000000}" name="Wk50 2025" dataDxfId="85"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0700-000022000000}" name="Wk51 2025" dataDxfId="84"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0700-000023000000}" name="Wk52 2025" dataDxfId="83"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0700-000024000000}" name="Wk 1 2026" dataDxfId="82"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0700-000025000000}" name="Wk 2 2026" dataDxfId="81"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0700-000026000000}" name="Wk 3 2026" dataDxfId="80"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0700-000027000000}" name="Wk 4 2026" dataDxfId="79"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0700-000028000000}" name="Wk 5 2026" dataDxfId="78"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0700-000029000000}" name="Wk 6 2026" dataDxfId="77"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0700-00002A000000}" name="Wk 7 2026" dataDxfId="76"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0700-00002B000000}" name="Wk 8 2026" dataDxfId="75"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0700-00002C000000}" name="Wk 9 2026" dataDxfId="74"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0700-00002D000000}" name="Wk 10 2026" dataDxfId="17"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0700-00002E000000}" name="Wk 11 2026" dataDxfId="16"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0700-00002F000000}" name="Wk 12 2026" dataDxfId="15"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0700-000030000000}" name="Wk 13 2026" dataDxfId="14"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0700-000031000000}" name="Wk 14 2026" dataDxfId="13"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0700-000032000000}" name="Wk 15 2026" dataDxfId="12"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0700-000033000000}" name="Wk 16 2026" dataDxfId="11"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0700-000034000000}" name="Wk 17 2026" dataDxfId="10"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0700-000035000000}" name="Wk 18 2026" dataDxfId="9"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0700-000036000000}" name="Wk 19 2026" dataDxfId="73"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0700-000037000000}" name="Wk 20 2026" dataDxfId="72"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0700-000038000000}" name="Wk 21 2026" dataDxfId="71"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0700-000039000000}" name="Wk 22 2026" dataDxfId="70"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0700-00003A000000}" name="Wk 23 2026" dataDxfId="69"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0700-00003B000000}" name="Wk 24 2026" dataDxfId="68"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0700-00003C000000}" name="Wk 25 2026" dataDxfId="67"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0700-00003D000000}" name="Wk 26 2026" dataDxfId="66"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0700-00003E000000}" name="Wk 27 2026" dataDxfId="65"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0700-00003F000000}" name="Wk 28 2026" dataDxfId="64"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0700-000040000000}" name="Wk 29 2026" dataDxfId="63"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0700-000041000000}" name="Wk 30 2026" dataDxfId="62"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0700-000042000000}" name="Wk 31 2026" dataDxfId="61"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0700-000043000000}" name="Wk 32 2026" dataDxfId="60"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0700-000044000000}" name="Wk 33 2026" dataDxfId="59"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0700-000045000000}" name="Wk 34 2026" dataDxfId="58"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0700-000046000000}" name="Wk 35 2026" dataDxfId="57"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0700-000047000000}" name="Wk 36 2026" dataDxfId="56"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0700-000048000000}" name="Wk 37 2026" dataDxfId="55"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0700-000049000000}" name="Wk 38 2026" dataDxfId="54"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0700-00004A000000}" name="Wk 39 2026" dataDxfId="53"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0700-00004B000000}" name="Wk 40 2026" dataDxfId="52"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0700-00004C000000}" name="Wk 41 2026" dataDxfId="51"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0700-00004D000000}" name="Wk 42 2026" dataDxfId="50"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0700-00004E000000}" name="Wk 43 2026" dataDxfId="49"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0700-00004F000000}" name="Wk 44 2026" dataDxfId="48"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0700-000050000000}" name="Wk 45 2026" dataDxfId="47"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0700-000051000000}" name="Wk 46 2026" dataDxfId="46"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0700-000052000000}" name="Wk 47 2026" dataDxfId="45"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0700-000053000000}" name="Wk 48 2026" dataDxfId="44"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0700-000054000000}" name="Wk 49 2026" dataDxfId="43"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0700-000055000000}" name="Wk 50 2026" dataDxfId="42"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0700-000056000000}" name="Wk 51 2026" dataDxfId="41"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0700-000057000000}" name="Wk 52 2026" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -27030,7 +27028,7 @@
       <c r="X4" s="37"/>
       <c r="Y4" s="37"/>
       <c r="Z4" s="1">
-        <f t="shared" ref="Z4:AT4" si="0">Z15*Z26*Z37</f>
+        <f t="shared" ref="Z4:BB7" si="0">Z15*Z26*Z37</f>
         <v>69096.999999999782</v>
       </c>
       <c r="AA4" s="1">
@@ -27110,17 +27108,32 @@
         <v>265183.0463662087</v>
       </c>
       <c r="AT4" s="1">
-        <f t="shared" si="0"/>
-        <v>331822.5846242765</v>
-      </c>
-      <c r="AU4" s="52"/>
-      <c r="AV4" s="52"/>
-      <c r="AW4" s="52"/>
-      <c r="AX4" s="52"/>
-      <c r="AY4" s="52"/>
-      <c r="AZ4" s="52"/>
-      <c r="BA4" s="52"/>
-      <c r="BB4" s="52"/>
+        <v>314053.97268299997</v>
+      </c>
+      <c r="AU4" s="52">
+        <v>426939.12572636135</v>
+      </c>
+      <c r="AV4" s="52">
+        <v>391450.88641064521</v>
+      </c>
+      <c r="AW4" s="52">
+        <v>307166.87101255532</v>
+      </c>
+      <c r="AX4" s="52">
+        <v>365866.11738837097</v>
+      </c>
+      <c r="AY4" s="52">
+        <v>322413.59259159508</v>
+      </c>
+      <c r="AZ4" s="52">
+        <v>394647.26686109503</v>
+      </c>
+      <c r="BA4" s="52">
+        <v>318938.37379659509</v>
+      </c>
+      <c r="BB4" s="52">
+        <v>306288.13428622007</v>
+      </c>
       <c r="BC4" s="52"/>
       <c r="BD4" s="52"/>
       <c r="BE4" s="52"/>
@@ -27264,17 +27277,32 @@
         <v>102515.03102087471</v>
       </c>
       <c r="AT5" s="1">
-        <f t="shared" si="1"/>
-        <v>128102.31679247835</v>
-      </c>
-      <c r="AU5" s="2"/>
-      <c r="AV5" s="2"/>
-      <c r="AW5" s="2"/>
-      <c r="AX5" s="2"/>
-      <c r="AY5" s="2"/>
-      <c r="AZ5" s="2"/>
-      <c r="BA5" s="2"/>
-      <c r="BB5" s="2"/>
+        <v>67843.7527348</v>
+      </c>
+      <c r="AU5" s="2">
+        <v>105976.89323418366</v>
+      </c>
+      <c r="AV5" s="2">
+        <v>96278.496868551505</v>
+      </c>
+      <c r="AW5" s="2">
+        <v>69995.868917128901</v>
+      </c>
+      <c r="AX5" s="2">
+        <v>90682.014134647703</v>
+      </c>
+      <c r="AY5" s="2">
+        <v>80409.456954096007</v>
+      </c>
+      <c r="AZ5" s="2">
+        <v>93566.659404717604</v>
+      </c>
+      <c r="BA5" s="2">
+        <v>79625.462824544302</v>
+      </c>
+      <c r="BB5" s="2">
+        <v>80865.876847471009</v>
+      </c>
       <c r="BC5" s="2"/>
       <c r="BD5" s="2"/>
       <c r="BE5" s="2"/>
@@ -27418,17 +27446,32 @@
         <v>39680.887413488483</v>
       </c>
       <c r="AT6" s="1">
-        <f t="shared" si="2"/>
-        <v>64711.901031597794</v>
-      </c>
-      <c r="AU6" s="2"/>
-      <c r="AV6" s="2"/>
-      <c r="AW6" s="2"/>
-      <c r="AX6" s="2"/>
-      <c r="AY6" s="2"/>
-      <c r="AZ6" s="2"/>
-      <c r="BA6" s="2"/>
-      <c r="BB6" s="2"/>
+        <v>21167.970328618107</v>
+      </c>
+      <c r="AU6" s="2">
+        <v>47990.985000000001</v>
+      </c>
+      <c r="AV6" s="2">
+        <v>47772.448815999996</v>
+      </c>
+      <c r="AW6" s="2">
+        <v>19610.154432000003</v>
+      </c>
+      <c r="AX6" s="2">
+        <v>22209.137280000003</v>
+      </c>
+      <c r="AY6" s="2">
+        <v>21723.988968000005</v>
+      </c>
+      <c r="AZ6" s="2">
+        <v>22211.197272000001</v>
+      </c>
+      <c r="BA6" s="2">
+        <v>21821.374080000001</v>
+      </c>
+      <c r="BB6" s="2">
+        <v>22343.077152000002</v>
+      </c>
       <c r="BC6" s="2"/>
       <c r="BD6" s="2"/>
       <c r="BE6" s="2"/>
@@ -27572,17 +27615,32 @@
         <v>97916.117131298859</v>
       </c>
       <c r="AT7" s="1">
-        <f t="shared" si="3"/>
-        <v>138707.27898055236</v>
-      </c>
-      <c r="AU7" s="2"/>
-      <c r="AV7" s="2"/>
-      <c r="AW7" s="2"/>
-      <c r="AX7" s="2"/>
-      <c r="AY7" s="2"/>
-      <c r="AZ7" s="2"/>
-      <c r="BA7" s="2"/>
-      <c r="BB7" s="2"/>
+        <v>123046.22632425652</v>
+      </c>
+      <c r="AU7" s="2">
+        <v>142544.66855199999</v>
+      </c>
+      <c r="AV7" s="2">
+        <v>138011.70648245353</v>
+      </c>
+      <c r="AW7" s="2">
+        <v>109061.35424786006</v>
+      </c>
+      <c r="AX7" s="2">
+        <v>93002.069373721897</v>
+      </c>
+      <c r="AY7" s="2">
+        <v>89829.984830617192</v>
+      </c>
+      <c r="AZ7" s="2">
+        <v>101786.31525431247</v>
+      </c>
+      <c r="BA7" s="2">
+        <v>94820.247495503078</v>
+      </c>
+      <c r="BB7" s="2">
+        <v>95681.314234902457</v>
+      </c>
       <c r="BC7" s="2"/>
       <c r="BD7" s="2"/>
       <c r="BE7" s="2"/>
@@ -27646,7 +27704,7 @@
       <c r="X8" s="37"/>
       <c r="Y8" s="37"/>
       <c r="Z8" s="1">
-        <f t="shared" ref="Z8:AT8" si="4">Z19*Z30*Z41</f>
+        <f t="shared" ref="Z8:BB8" si="4">Z19*Z30*Z41</f>
         <v>3516.9999999999741</v>
       </c>
       <c r="AA8" s="1">
@@ -27726,17 +27784,32 @@
         <v>54227.654056660394</v>
       </c>
       <c r="AT8" s="1">
-        <f t="shared" si="4"/>
-        <v>120678.20308585466</v>
-      </c>
-      <c r="AU8" s="2"/>
-      <c r="AV8" s="2"/>
-      <c r="AW8" s="2"/>
-      <c r="AX8" s="2"/>
-      <c r="AY8" s="2"/>
-      <c r="AZ8" s="2"/>
-      <c r="BA8" s="2"/>
-      <c r="BB8" s="2"/>
+        <v>130209.59537543617</v>
+      </c>
+      <c r="AU8" s="2">
+        <v>131241.58316399998</v>
+      </c>
+      <c r="AV8" s="2">
+        <v>127331.36149724819</v>
+      </c>
+      <c r="AW8" s="2">
+        <v>99243.168388601931</v>
+      </c>
+      <c r="AX8" s="2">
+        <v>95746.03420740529</v>
+      </c>
+      <c r="AY8" s="2">
+        <v>113039.15319763083</v>
+      </c>
+      <c r="AZ8" s="2">
+        <v>113656.96290926401</v>
+      </c>
+      <c r="BA8" s="2">
+        <v>117981.05337869808</v>
+      </c>
+      <c r="BB8" s="2">
+        <v>119558.07888248673</v>
+      </c>
       <c r="BC8" s="2"/>
       <c r="BD8" s="2"/>
       <c r="BE8" s="2"/>
@@ -27800,7 +27873,7 @@
       <c r="X9" s="37"/>
       <c r="Y9" s="37"/>
       <c r="Z9" s="1">
-        <f t="shared" ref="Z9:AT9" si="5">SUBTOTAL(109,Z4:Z8)</f>
+        <f t="shared" ref="Z9:BB9" si="5">SUBTOTAL(109,Z4:Z8)</f>
         <v>124123.99999999968</v>
       </c>
       <c r="AA9" s="1">
@@ -27880,17 +27953,32 @@
         <v>559522.73598853115</v>
       </c>
       <c r="AT9" s="1">
-        <f t="shared" si="5"/>
-        <v>784022.28451475955</v>
-      </c>
-      <c r="AU9" s="51"/>
-      <c r="AV9" s="51"/>
-      <c r="AW9" s="51"/>
-      <c r="AX9" s="51"/>
-      <c r="AY9" s="51"/>
-      <c r="AZ9" s="51"/>
-      <c r="BA9" s="51"/>
-      <c r="BB9" s="51"/>
+        <v>656321.51744611072</v>
+      </c>
+      <c r="AU9" s="51">
+        <v>854693.25567654497</v>
+      </c>
+      <c r="AV9" s="51">
+        <v>800844.90007489838</v>
+      </c>
+      <c r="AW9" s="51">
+        <v>605077.41699814622</v>
+      </c>
+      <c r="AX9" s="51">
+        <v>667505.37238414586</v>
+      </c>
+      <c r="AY9" s="51">
+        <v>627416.17654193914</v>
+      </c>
+      <c r="AZ9" s="51">
+        <v>725868.40170138911</v>
+      </c>
+      <c r="BA9" s="51">
+        <v>633186.51157534053</v>
+      </c>
+      <c r="BB9" s="51">
+        <v>624736.48140308028</v>
+      </c>
       <c r="BC9" s="51"/>
       <c r="BD9" s="51"/>
       <c r="BE9" s="51"/>
@@ -28329,16 +28417,32 @@
         <v>1181576.422222222</v>
       </c>
       <c r="AT15" s="2">
-        <v>1221902.722222222</v>
-      </c>
-      <c r="AU15" s="50"/>
-      <c r="AV15" s="50"/>
-      <c r="AW15" s="50"/>
-      <c r="AX15" s="50"/>
-      <c r="AY15" s="50"/>
-      <c r="AZ15" s="50"/>
-      <c r="BA15" s="50"/>
-      <c r="BB15" s="50"/>
+        <v>1464571.7222222222</v>
+      </c>
+      <c r="AU15" s="50">
+        <v>1824175.3753609834</v>
+      </c>
+      <c r="AV15" s="50">
+        <v>1679325.9820276499</v>
+      </c>
+      <c r="AW15" s="50">
+        <v>1450001.5153609831</v>
+      </c>
+      <c r="AX15" s="50">
+        <v>1721220.7139016897</v>
+      </c>
+      <c r="AY15" s="50">
+        <v>1521974.672235023</v>
+      </c>
+      <c r="AZ15" s="50">
+        <v>1862958.5055683563</v>
+      </c>
+      <c r="BA15" s="50">
+        <v>1505569.672235023</v>
+      </c>
+      <c r="BB15" s="50">
+        <v>1445853.3805683563</v>
+      </c>
       <c r="BC15" s="50"/>
       <c r="BD15" s="50"/>
       <c r="BE15" s="50"/>
@@ -28462,16 +28566,32 @@
         <v>1094551.771804444</v>
       </c>
       <c r="AT16" s="1">
-        <v>1130369.3544444451</v>
-      </c>
-      <c r="AU16" s="49"/>
-      <c r="AV16" s="49"/>
-      <c r="AW16" s="49"/>
-      <c r="AX16" s="49"/>
-      <c r="AY16" s="49"/>
-      <c r="AZ16" s="49"/>
-      <c r="BA16" s="49"/>
-      <c r="BB16" s="49"/>
+        <v>1405855.0444444446</v>
+      </c>
+      <c r="AU16" s="49">
+        <v>1734482.7043237917</v>
+      </c>
+      <c r="AV16" s="49">
+        <v>1587967.9509904585</v>
+      </c>
+      <c r="AW16" s="49">
+        <v>1450511.2093237918</v>
+      </c>
+      <c r="AX16" s="49">
+        <v>1849898.2891605</v>
+      </c>
+      <c r="AY16" s="49">
+        <v>1644667.8724938333</v>
+      </c>
+      <c r="AZ16" s="49">
+        <v>1923933.5308271667</v>
+      </c>
+      <c r="BA16" s="49">
+        <v>1632940.8724938333</v>
+      </c>
+      <c r="BB16" s="49">
+        <v>1654003.3308271668</v>
+      </c>
       <c r="BC16" s="49"/>
       <c r="BD16" s="49"/>
       <c r="BE16" s="49"/>
@@ -28595,16 +28715,32 @@
         <v>592436.3157999533</v>
       </c>
       <c r="AT17" s="1">
-        <v>798470.88403995335</v>
-      </c>
-      <c r="AU17" s="49"/>
-      <c r="AV17" s="49"/>
-      <c r="AW17" s="49"/>
-      <c r="AX17" s="49"/>
-      <c r="AY17" s="49"/>
-      <c r="AZ17" s="49"/>
-      <c r="BA17" s="49"/>
-      <c r="BB17" s="49"/>
+        <v>522665.93403995328</v>
+      </c>
+      <c r="AU17" s="49">
+        <v>457057</v>
+      </c>
+      <c r="AV17" s="49">
+        <v>492662</v>
+      </c>
+      <c r="AW17" s="49">
+        <v>485496</v>
+      </c>
+      <c r="AX17" s="49">
+        <v>549840</v>
+      </c>
+      <c r="AY17" s="49">
+        <v>537829</v>
+      </c>
+      <c r="AZ17" s="49">
+        <v>549891</v>
+      </c>
+      <c r="BA17" s="49">
+        <v>540240</v>
+      </c>
+      <c r="BB17" s="49">
+        <v>553156</v>
+      </c>
       <c r="BC17" s="49"/>
       <c r="BD17" s="49"/>
       <c r="BE17" s="49"/>
@@ -28728,16 +28864,32 @@
         <v>1025090.713887653</v>
       </c>
       <c r="AT18" s="1">
-        <v>1200112.607407653</v>
-      </c>
-      <c r="AU18" s="49"/>
-      <c r="AV18" s="49"/>
-      <c r="AW18" s="49"/>
-      <c r="AX18" s="49"/>
-      <c r="AY18" s="49"/>
-      <c r="AZ18" s="49"/>
-      <c r="BA18" s="49"/>
-      <c r="BB18" s="49"/>
+        <v>1304810.3574076532</v>
+      </c>
+      <c r="AU18" s="49">
+        <v>1457989</v>
+      </c>
+      <c r="AV18" s="49">
+        <v>1409879.6236804293</v>
+      </c>
+      <c r="AW18" s="49">
+        <v>1310455.5686804294</v>
+      </c>
+      <c r="AX18" s="49">
+        <v>1186614.1340936241</v>
+      </c>
+      <c r="AY18" s="49">
+        <v>1122987.1090936242</v>
+      </c>
+      <c r="AZ18" s="49">
+        <v>1247259.0340936242</v>
+      </c>
+      <c r="BA18" s="49">
+        <v>1117636.1090936242</v>
+      </c>
+      <c r="BB18" s="49">
+        <v>1087745.0090936241</v>
+      </c>
       <c r="BC18" s="49"/>
       <c r="BD18" s="49"/>
       <c r="BE18" s="49"/>
@@ -28861,16 +29013,32 @@
         <v>673962.98136297008</v>
       </c>
       <c r="AT19" s="1">
-        <v>859028.5405629701</v>
-      </c>
-      <c r="AU19" s="49"/>
-      <c r="AV19" s="49"/>
-      <c r="AW19" s="49"/>
-      <c r="AX19" s="49"/>
-      <c r="AY19" s="49"/>
-      <c r="AZ19" s="49"/>
-      <c r="BA19" s="49"/>
-      <c r="BB19" s="49"/>
+        <v>950074.39056297007</v>
+      </c>
+      <c r="AU19" s="49">
+        <v>1053743</v>
+      </c>
+      <c r="AV19" s="49">
+        <v>1029289.6295894217</v>
+      </c>
+      <c r="AW19" s="49">
+        <v>961854.33458942163</v>
+      </c>
+      <c r="AX19" s="49">
+        <v>1019789.9008116618</v>
+      </c>
+      <c r="AY19" s="49">
+        <v>958161.92581166187</v>
+      </c>
+      <c r="AZ19" s="49">
+        <v>1049929.4508116618</v>
+      </c>
+      <c r="BA19" s="49">
+        <v>970238.92581166187</v>
+      </c>
+      <c r="BB19" s="49">
+        <v>940210.27581166185</v>
+      </c>
       <c r="BC19" s="49"/>
       <c r="BD19" s="49"/>
       <c r="BE19" s="49"/>
@@ -29014,17 +29182,32 @@
         <v>4567618.2050772421</v>
       </c>
       <c r="AT20" s="2">
-        <f t="shared" si="6"/>
         <v>5209884.1086772438</v>
       </c>
-      <c r="AU20" s="48"/>
-      <c r="AV20" s="48"/>
-      <c r="AW20" s="48"/>
-      <c r="AX20" s="48"/>
-      <c r="AY20" s="48"/>
-      <c r="AZ20" s="48"/>
-      <c r="BA20" s="48"/>
-      <c r="BB20" s="48"/>
+      <c r="AU20" s="48">
+        <v>6527447.0796847753</v>
+      </c>
+      <c r="AV20" s="48">
+        <v>6199125.1862879591</v>
+      </c>
+      <c r="AW20" s="48">
+        <v>5658318.6279546265</v>
+      </c>
+      <c r="AX20" s="48">
+        <v>6327363.0379674761</v>
+      </c>
+      <c r="AY20" s="48">
+        <v>5785620.579634143</v>
+      </c>
+      <c r="AZ20" s="48">
+        <v>6633971.5213008085</v>
+      </c>
+      <c r="BA20" s="48">
+        <v>5766625.579634143</v>
+      </c>
+      <c r="BB20" s="48">
+        <v>5680967.9963008091</v>
+      </c>
       <c r="BC20" s="48"/>
       <c r="BD20" s="48"/>
       <c r="BE20" s="48"/>
@@ -29416,16 +29599,32 @@
         <v>2.5582525859249351E-2</v>
       </c>
       <c r="AT26" s="47">
-        <v>2.8140778445174291E-2</v>
-      </c>
-      <c r="AU26" s="47"/>
-      <c r="AV26" s="47"/>
-      <c r="AW26" s="47"/>
-      <c r="AX26" s="47"/>
-      <c r="AY26" s="47"/>
-      <c r="AZ26" s="47"/>
-      <c r="BA26" s="47"/>
-      <c r="BB26" s="47"/>
+        <v>2.9700000000000001E-2</v>
+      </c>
+      <c r="AU26" s="47">
+        <v>3.15E-2</v>
+      </c>
+      <c r="AV26" s="47">
+        <v>3.15E-2</v>
+      </c>
+      <c r="AW26" s="47">
+        <v>2.93E-2</v>
+      </c>
+      <c r="AX26" s="47">
+        <v>2.9399999999999999E-2</v>
+      </c>
+      <c r="AY26" s="47">
+        <v>2.93E-2</v>
+      </c>
+      <c r="AZ26" s="47">
+        <v>2.93E-2</v>
+      </c>
+      <c r="BA26" s="47">
+        <v>2.93E-2</v>
+      </c>
+      <c r="BB26" s="47">
+        <v>2.93E-2</v>
+      </c>
       <c r="BC26" s="47"/>
       <c r="BD26" s="47"/>
       <c r="BE26" s="47"/>
@@ -29549,16 +29748,32 @@
         <v>1.6665091291966781E-2</v>
       </c>
       <c r="AT27" s="46">
-        <v>1.8331600421163469E-2</v>
-      </c>
-      <c r="AU27" s="46"/>
-      <c r="AV27" s="46"/>
-      <c r="AW27" s="46"/>
-      <c r="AX27" s="46"/>
-      <c r="AY27" s="46"/>
-      <c r="AZ27" s="46"/>
-      <c r="BA27" s="46"/>
-      <c r="BB27" s="46"/>
+        <v>1.26E-2</v>
+      </c>
+      <c r="AU27" s="46">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="AV27" s="46">
+        <v>1.29E-2</v>
+      </c>
+      <c r="AW27" s="46">
+        <v>1.2800000000000001E-2</v>
+      </c>
+      <c r="AX27" s="46">
+        <v>1.29E-2</v>
+      </c>
+      <c r="AY27" s="46">
+        <v>1.29E-2</v>
+      </c>
+      <c r="AZ27" s="46">
+        <v>1.29E-2</v>
+      </c>
+      <c r="BA27" s="46">
+        <v>1.29E-2</v>
+      </c>
+      <c r="BB27" s="46">
+        <v>1.29E-2</v>
+      </c>
       <c r="BC27" s="46"/>
       <c r="BD27" s="46"/>
       <c r="BE27" s="46"/>
@@ -29682,16 +29897,32 @@
         <v>9.0903399389920484E-3</v>
       </c>
       <c r="AT28" s="46">
-        <v>9.9993739328912545E-3</v>
-      </c>
-      <c r="AU28" s="46"/>
-      <c r="AV28" s="46"/>
-      <c r="AW28" s="46"/>
-      <c r="AX28" s="46"/>
-      <c r="AY28" s="46"/>
-      <c r="AZ28" s="46"/>
-      <c r="BA28" s="46"/>
-      <c r="BB28" s="46"/>
+        <v>0.01</v>
+      </c>
+      <c r="AU28" s="46">
+        <v>1.4E-2</v>
+      </c>
+      <c r="AV28" s="46">
+        <v>1.3599999999999999E-2</v>
+      </c>
+      <c r="AW28" s="46">
+        <v>9.9000000000000008E-3</v>
+      </c>
+      <c r="AX28" s="46">
+        <v>9.9000000000000008E-3</v>
+      </c>
+      <c r="AY28" s="46">
+        <v>9.9000000000000008E-3</v>
+      </c>
+      <c r="AZ28" s="46">
+        <v>9.9000000000000008E-3</v>
+      </c>
+      <c r="BA28" s="46">
+        <v>9.9000000000000008E-3</v>
+      </c>
+      <c r="BB28" s="46">
+        <v>9.9000000000000008E-3</v>
+      </c>
       <c r="BC28" s="46"/>
       <c r="BD28" s="46"/>
       <c r="BE28" s="46"/>
@@ -29815,16 +30046,32 @@
         <v>1.1086078152387289E-2</v>
       </c>
       <c r="AT29" s="46">
-        <v>1.2194685967626019E-2</v>
-      </c>
-      <c r="AU29" s="46"/>
-      <c r="AV29" s="46"/>
-      <c r="AW29" s="46"/>
-      <c r="AX29" s="46"/>
-      <c r="AY29" s="46"/>
-      <c r="AZ29" s="46"/>
-      <c r="BA29" s="46"/>
-      <c r="BB29" s="46"/>
+        <v>1.17E-2</v>
+      </c>
+      <c r="AU29" s="46">
+        <v>1.21E-2</v>
+      </c>
+      <c r="AV29" s="46">
+        <v>1.21E-2</v>
+      </c>
+      <c r="AW29" s="46">
+        <v>1.03E-2</v>
+      </c>
+      <c r="AX29" s="46">
+        <v>9.7000000000000003E-3</v>
+      </c>
+      <c r="AY29" s="46">
+        <v>9.9000000000000008E-3</v>
+      </c>
+      <c r="AZ29" s="46">
+        <v>1.01E-2</v>
+      </c>
+      <c r="BA29" s="46">
+        <v>1.0500000000000001E-2</v>
+      </c>
+      <c r="BB29" s="46">
+        <v>1.09E-2</v>
+      </c>
       <c r="BC29" s="46"/>
       <c r="BD29" s="46"/>
       <c r="BE29" s="46"/>
@@ -29948,16 +30195,32 @@
         <v>1.0395375027810761E-2</v>
       </c>
       <c r="AT30" s="46">
+        <v>2.4299999999999999E-2</v>
+      </c>
+      <c r="AU30" s="46">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="AV30" s="46">
+        <v>1.83E-2</v>
+      </c>
+      <c r="AW30" s="46">
+        <v>1.6299999999999999E-2</v>
+      </c>
+      <c r="AX30" s="46">
+        <v>1.44E-2</v>
+      </c>
+      <c r="AY30" s="46">
         <v>1.6500000000000001E-2</v>
       </c>
-      <c r="AU30" s="46"/>
-      <c r="AV30" s="46"/>
-      <c r="AW30" s="46"/>
-      <c r="AX30" s="46"/>
-      <c r="AY30" s="46"/>
-      <c r="AZ30" s="46"/>
-      <c r="BA30" s="46"/>
-      <c r="BB30" s="46"/>
+      <c r="AZ30" s="46">
+        <v>1.8599999999999998E-2</v>
+      </c>
+      <c r="BA30" s="46">
+        <v>0.02</v>
+      </c>
+      <c r="BB30" s="46">
+        <v>2.1299999999999999E-2</v>
+      </c>
       <c r="BC30" s="46"/>
       <c r="BD30" s="46"/>
       <c r="BE30" s="46"/>
@@ -30101,17 +30364,32 @@
         <v>1.5812244489524521E-2</v>
       </c>
       <c r="AT31" s="45">
-        <f t="shared" si="7"/>
-        <v>1.7639538124275798E-2</v>
-      </c>
-      <c r="AU31" s="44"/>
-      <c r="AV31" s="44"/>
-      <c r="AW31" s="44"/>
-      <c r="AX31" s="44"/>
-      <c r="AY31" s="44"/>
-      <c r="AZ31" s="44"/>
-      <c r="BA31" s="44"/>
-      <c r="BB31" s="44"/>
+        <v>2.0113941066024037E-2</v>
+      </c>
+      <c r="AU31" s="44">
+        <v>1.9395080961145696E-2</v>
+      </c>
+      <c r="AV31" s="44">
+        <v>1.8708978829175087E-2</v>
+      </c>
+      <c r="AW31" s="44">
+        <v>1.6795433862831131E-2</v>
+      </c>
+      <c r="AX31" s="44">
+        <v>1.6769406774130732E-2</v>
+      </c>
+      <c r="AY31" s="44">
+        <v>1.6949231868533091E-2</v>
+      </c>
+      <c r="AZ31" s="44">
+        <v>1.7632477214392581E-2</v>
+      </c>
+      <c r="BA31" s="44">
+        <v>1.7630147979856015E-2</v>
+      </c>
+      <c r="BB31" s="44">
+        <v>1.7789097026780904E-2</v>
+      </c>
       <c r="BC31" s="44"/>
       <c r="BD31" s="44"/>
       <c r="BE31" s="44"/>
@@ -30485,16 +30763,32 @@
         <v>8.7728462340975071</v>
       </c>
       <c r="AT37" s="42">
-        <v>9.6501308575072589</v>
-      </c>
-      <c r="AU37" s="42"/>
-      <c r="AV37" s="42"/>
-      <c r="AW37" s="42"/>
-      <c r="AX37" s="42"/>
-      <c r="AY37" s="42"/>
-      <c r="AZ37" s="42"/>
-      <c r="BA37" s="42"/>
-      <c r="BB37" s="42"/>
+        <v>7.22</v>
+      </c>
+      <c r="AU37" s="42">
+        <v>7.43</v>
+      </c>
+      <c r="AV37" s="42">
+        <v>7.4</v>
+      </c>
+      <c r="AW37" s="42">
+        <v>7.23</v>
+      </c>
+      <c r="AX37" s="42">
+        <v>7.23</v>
+      </c>
+      <c r="AY37" s="42">
+        <v>7.23</v>
+      </c>
+      <c r="AZ37" s="42">
+        <v>7.23</v>
+      </c>
+      <c r="BA37" s="42">
+        <v>7.23</v>
+      </c>
+      <c r="BB37" s="42">
+        <v>7.23</v>
+      </c>
       <c r="BC37" s="42"/>
       <c r="BD37" s="42"/>
       <c r="BE37" s="42"/>
@@ -30600,16 +30894,32 @@
         <v>5.6200935151584339</v>
       </c>
       <c r="AT38" s="41">
-        <v>6.1821028666742777</v>
-      </c>
-      <c r="AU38" s="41"/>
-      <c r="AV38" s="41"/>
-      <c r="AW38" s="41"/>
-      <c r="AX38" s="41"/>
-      <c r="AY38" s="41"/>
-      <c r="AZ38" s="41"/>
-      <c r="BA38" s="41"/>
-      <c r="BB38" s="41"/>
+        <v>3.83</v>
+      </c>
+      <c r="AU38" s="41">
+        <v>4.7</v>
+      </c>
+      <c r="AV38" s="41">
+        <v>4.7</v>
+      </c>
+      <c r="AW38" s="41">
+        <v>3.77</v>
+      </c>
+      <c r="AX38" s="41">
+        <v>3.8</v>
+      </c>
+      <c r="AY38" s="41">
+        <v>3.79</v>
+      </c>
+      <c r="AZ38" s="41">
+        <v>3.77</v>
+      </c>
+      <c r="BA38" s="41">
+        <v>3.78</v>
+      </c>
+      <c r="BB38" s="41">
+        <v>3.79</v>
+      </c>
       <c r="BC38" s="41"/>
       <c r="BD38" s="41"/>
       <c r="BE38" s="41"/>
@@ -30715,16 +31025,32 @@
         <v>7.3681690133770372</v>
       </c>
       <c r="AT39" s="41">
-        <v>8.1049859147147405</v>
-      </c>
-      <c r="AU39" s="41"/>
-      <c r="AV39" s="41"/>
-      <c r="AW39" s="41"/>
-      <c r="AX39" s="41"/>
-      <c r="AY39" s="41"/>
-      <c r="AZ39" s="41"/>
-      <c r="BA39" s="41"/>
-      <c r="BB39" s="41"/>
+        <v>4.05</v>
+      </c>
+      <c r="AU39" s="41">
+        <v>7.5</v>
+      </c>
+      <c r="AV39" s="41">
+        <v>7.13</v>
+      </c>
+      <c r="AW39" s="41">
+        <v>4.08</v>
+      </c>
+      <c r="AX39" s="41">
+        <v>4.08</v>
+      </c>
+      <c r="AY39" s="41">
+        <v>4.08</v>
+      </c>
+      <c r="AZ39" s="41">
+        <v>4.08</v>
+      </c>
+      <c r="BA39" s="41">
+        <v>4.08</v>
+      </c>
+      <c r="BB39" s="41">
+        <v>4.08</v>
+      </c>
       <c r="BC39" s="41"/>
       <c r="BD39" s="41"/>
       <c r="BE39" s="41"/>
@@ -30830,16 +31156,32 @@
         <v>8.6161638261499363</v>
       </c>
       <c r="AT40" s="41">
-        <v>9.4777802087649299</v>
-      </c>
-      <c r="AU40" s="41"/>
-      <c r="AV40" s="41"/>
-      <c r="AW40" s="41"/>
-      <c r="AX40" s="41"/>
-      <c r="AY40" s="41"/>
-      <c r="AZ40" s="41"/>
-      <c r="BA40" s="41"/>
-      <c r="BB40" s="41"/>
+        <v>8.06</v>
+      </c>
+      <c r="AU40" s="41">
+        <v>8.08</v>
+      </c>
+      <c r="AV40" s="41">
+        <v>8.09</v>
+      </c>
+      <c r="AW40" s="41">
+        <v>8.08</v>
+      </c>
+      <c r="AX40" s="41">
+        <v>8.08</v>
+      </c>
+      <c r="AY40" s="41">
+        <v>8.08</v>
+      </c>
+      <c r="AZ40" s="41">
+        <v>8.08</v>
+      </c>
+      <c r="BA40" s="41">
+        <v>8.08</v>
+      </c>
+      <c r="BB40" s="41">
+        <v>8.07</v>
+      </c>
       <c r="BC40" s="41"/>
       <c r="BD40" s="41"/>
       <c r="BE40" s="41"/>
@@ -30945,16 +31287,32 @@
         <v>7.740065079538069</v>
       </c>
       <c r="AT41" s="41">
-        <v>8.5140715874918769</v>
-      </c>
-      <c r="AU41" s="41"/>
-      <c r="AV41" s="41"/>
-      <c r="AW41" s="41"/>
-      <c r="AX41" s="41"/>
-      <c r="AY41" s="41"/>
-      <c r="AZ41" s="41"/>
-      <c r="BA41" s="41"/>
-      <c r="BB41" s="41"/>
+        <v>5.64</v>
+      </c>
+      <c r="AU41" s="41">
+        <v>5.82</v>
+      </c>
+      <c r="AV41" s="41">
+        <v>6.76</v>
+      </c>
+      <c r="AW41" s="41">
+        <v>6.33</v>
+      </c>
+      <c r="AX41" s="41">
+        <v>6.52</v>
+      </c>
+      <c r="AY41" s="41">
+        <v>7.15</v>
+      </c>
+      <c r="AZ41" s="41">
+        <v>5.82</v>
+      </c>
+      <c r="BA41" s="41">
+        <v>6.08</v>
+      </c>
+      <c r="BB41" s="41">
+        <v>5.97</v>
+      </c>
       <c r="BC41" s="41"/>
       <c r="BD41" s="41"/>
       <c r="BE41" s="41"/>
@@ -31000,7 +31358,7 @@
       <c r="L42" s="34"/>
       <c r="M42" s="34"/>
       <c r="Z42" s="39">
-        <f t="shared" ref="Z42:AT42" si="8">SUM(Z4:Z8)/SUMPRODUCT(Z15:Z19,Z26:Z30)</f>
+        <f t="shared" ref="Z42:BB42" si="8">SUM(Z4:Z8)/SUMPRODUCT(Z15:Z19,Z26:Z30)</f>
         <v>5.5048784814617679</v>
       </c>
       <c r="AA42" s="39">
@@ -31080,17 +31438,32 @@
         <v>7.7470154584602655</v>
       </c>
       <c r="AT42" s="39">
-        <f t="shared" si="8"/>
-        <v>8.5312591572816228</v>
-      </c>
-      <c r="AU42" s="38"/>
-      <c r="AV42" s="38"/>
-      <c r="AW42" s="38"/>
-      <c r="AX42" s="38"/>
-      <c r="AY42" s="38"/>
-      <c r="AZ42" s="38"/>
-      <c r="BA42" s="38"/>
-      <c r="BB42" s="38"/>
+        <v>6.2631297197733282</v>
+      </c>
+      <c r="AU42" s="38">
+        <v>6.751112119712058</v>
+      </c>
+      <c r="AV42" s="38">
+        <v>6.9050674315564784</v>
+      </c>
+      <c r="AW42" s="38">
+        <v>6.3669628761553838</v>
+      </c>
+      <c r="AX42" s="38">
+        <v>6.2909221777290947</v>
+      </c>
+      <c r="AY42" s="38">
+        <v>6.3981695059511488</v>
+      </c>
+      <c r="AZ42" s="38">
+        <v>6.2054167997461418</v>
+      </c>
+      <c r="BA42" s="38">
+        <v>6.2280765669177125</v>
+      </c>
+      <c r="BB42" s="38">
+        <v>6.1818807146518377</v>
+      </c>
       <c r="BC42" s="38"/>
       <c r="BD42" s="38"/>
       <c r="BE42" s="38"/>

</xml_diff>

<commit_message>
v2.6.0: Historic model backtest with promo uplift
</commit_message>
<xml_diff>
--- a/inputs_forecasting.xlsx
+++ b/inputs_forecasting.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fnachbar\forecasting_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0AF524-0874-4B95-A87B-B8D10E3CF522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF140FD-0D44-40D9-915C-6F542041D9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10140" yWindow="32280" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Actuals" sheetId="1" r:id="rId1"/>
@@ -782,1212 +782,6 @@
   <dxfs count="654">
     <dxf>
       <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF212121"/>
-        <name val="Amazon Ember"/>
-        <family val="2"/>
-      </font>
-      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF6F6F6"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -2126,6 +920,294 @@
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.##;\-#,##0.##"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -5653,6 +4735,294 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00%;\-#,##0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
@@ -7061,6 +6431,348 @@
         <shadow val="0"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
         <color rgb="FF212121"/>
         <name val="Amazon Ember"/>
         <family val="2"/>
@@ -9915,6 +9627,294 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="12"/>
+        <color rgb="FF212121"/>
+        <name val="Amazon Ember"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF6F6F6"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
@@ -11615,6 +11615,7 @@
         <color rgb="FF212121"/>
         <name val="Amazon Ember"/>
         <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="14" formatCode="0.00%"/>
       <fill>
@@ -11623,20 +11624,22 @@
           <bgColor rgb="FFF6F6F6"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -14239,6 +14242,7 @@
         <color rgb="FF212121"/>
         <name val="Amazon Ember"/>
         <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
       <fill>
@@ -14247,8 +14251,8 @@
           <bgColor rgb="FFF6F6F6"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -16723,6 +16727,7 @@
         <color rgb="FF212121"/>
         <name val="Amazon Ember"/>
         <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="7" formatCode="#,##0.00;\-#,##0.00"/>
       <fill>
@@ -16731,20 +16736,22 @@
           <bgColor rgb="FFF6F6F6"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -19278,6 +19285,7 @@
         <color rgb="FF212121"/>
         <name val="Amazon Ember"/>
         <family val="2"/>
+        <scheme val="none"/>
       </font>
       <numFmt numFmtId="5" formatCode="#,##0;\-#,##0"/>
       <fill>
@@ -19286,8 +19294,8 @@
           <bgColor rgb="FFF6F6F6"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -20827,8 +20835,8 @@
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Wk 3 2026" dataDxfId="617"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Wk 4 2026" dataDxfId="616"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Wk 5 2026" dataDxfId="615"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Wk 6 2026" dataDxfId="39"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="Wk 7 2026" dataDxfId="614"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Wk 6 2026" dataDxfId="614"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="Wk 7 2026" dataDxfId="3"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="Wk 8 2026" dataDxfId="613"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="Wk 9 2026" dataDxfId="612"/>
     <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="Wk 10 2026" dataDxfId="611"/>
@@ -20927,8 +20935,8 @@
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0100-000026000000}" name="Wk 3 2026" dataDxfId="546"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0100-000027000000}" name="Wk 4 2026" dataDxfId="545"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0100-000028000000}" name="Wk 5 2026" dataDxfId="544"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0100-000029000000}" name="Wk 6 2026" dataDxfId="36"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0100-00002A000000}" name="Wk 7 2026" dataDxfId="543"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0100-000029000000}" name="Wk 6 2026" dataDxfId="543"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0100-00002A000000}" name="Wk 7 2026" dataDxfId="0"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0100-00002B000000}" name="Wk 8 2026" dataDxfId="542"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0100-00002C000000}" name="Wk 9 2026" dataDxfId="541"/>
     <tableColumn id="45" xr3:uid="{00000000-0010-0000-0100-00002D000000}" name="Wk 10 2026" dataDxfId="540"/>
@@ -21023,8 +21031,8 @@
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0200-000026000000}" name="Wk 3 2026" dataDxfId="476"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0200-000027000000}" name="Wk 4 2026" dataDxfId="475"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0200-000028000000}" name="Wk 5 2026" dataDxfId="474"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0200-000029000000}" name="Wk 6 2026" dataDxfId="38"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0200-00002A000000}" name="Wk 7 2026" dataDxfId="473"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0200-000029000000}" name="Wk 6 2026" dataDxfId="473"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0200-00002A000000}" name="Wk 7 2026" dataDxfId="2"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0200-00002B000000}" name="Wk 8 2026" dataDxfId="472"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0200-00002C000000}" name="Wk 9 2026" dataDxfId="471"/>
     <tableColumn id="45" xr3:uid="{00000000-0010-0000-0200-00002D000000}" name="Wk 10 2026" dataDxfId="470"/>
@@ -21119,8 +21127,8 @@
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0300-000026000000}" name="Wk 3 2026" dataDxfId="388" dataCellStyle="Percent"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0300-000027000000}" name="Wk 4 2026" dataDxfId="387" dataCellStyle="Percent"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0300-000028000000}" name="Wk 5 2026" dataDxfId="386" dataCellStyle="Percent"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0300-000029000000}" name="Wk 6 2026" dataDxfId="37" dataCellStyle="Percent"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0300-00002A000000}" name="Wk 7 2026" dataDxfId="385" dataCellStyle="Percent"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0300-000029000000}" name="Wk 6 2026" dataDxfId="385" dataCellStyle="Percent"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0300-00002A000000}" name="Wk 7 2026" dataDxfId="1" dataCellStyle="Percent"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0300-00002B000000}" name="Wk 8 2026" dataDxfId="384" dataCellStyle="Percent"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0300-00002C000000}" name="Wk 9 2026" dataDxfId="383" dataCellStyle="Percent"/>
     <tableColumn id="45" xr3:uid="{00000000-0010-0000-0300-00002D000000}" name="Wk 10 2026" dataDxfId="382" dataCellStyle="Percent"/>
@@ -21240,262 +21248,262 @@
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0400-00002C000000}" name="Wk 9 2026" dataDxfId="297">
       <calculatedColumnFormula>AS15*AS26*AS37</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0400-00002D000000}" name="Wk 10 2026" dataDxfId="8"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0400-00002E000000}" name="Wk 11 2026" dataDxfId="7"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0400-00002F000000}" name="Wk 12 2026" dataDxfId="6"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0400-000030000000}" name="Wk 13 2026" dataDxfId="5"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0400-000031000000}" name="Wk 14 2026" dataDxfId="4"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0400-000032000000}" name="Wk 15 2026" dataDxfId="3"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0400-000033000000}" name="Wk 16 2026" dataDxfId="2"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0400-000034000000}" name="Wk 17 2026" dataDxfId="1"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0400-000035000000}" name="Wk 18 2026" dataDxfId="0"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0400-000036000000}" name="Wk 19 2026" dataDxfId="296"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0400-000037000000}" name="Wk 20 2026" dataDxfId="295"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0400-000038000000}" name="Wk 21 2026" dataDxfId="294"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0400-000039000000}" name="Wk 22 2026" dataDxfId="293"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0400-00003A000000}" name="Wk 23 2026" dataDxfId="292"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0400-00003B000000}" name="Wk 24 2026" dataDxfId="291"/>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0400-00003C000000}" name="Wk 25 2026" dataDxfId="290"/>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0400-00003D000000}" name="Wk 26 2026" dataDxfId="289"/>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0400-00003E000000}" name="Wk 27 2026" dataDxfId="288"/>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0400-00003F000000}" name="Wk 28 2026" dataDxfId="287"/>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0400-000040000000}" name="Wk 29 2026" dataDxfId="286"/>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0400-000041000000}" name="Wk 30 2026" dataDxfId="285"/>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0400-000042000000}" name="Wk 31 2026" dataDxfId="284"/>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0400-000043000000}" name="Wk 32 2026" dataDxfId="283"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0400-000044000000}" name="Wk 33 2026" dataDxfId="282"/>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0400-000045000000}" name="Wk 34 2026" dataDxfId="281"/>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0400-000046000000}" name="Wk 35 2026" dataDxfId="280"/>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0400-000047000000}" name="Wk 36 2026" dataDxfId="279"/>
-    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0400-000048000000}" name="Wk 37 2026" dataDxfId="278"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0400-000049000000}" name="Wk 38 2026" dataDxfId="277"/>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0400-00004A000000}" name="Wk 39 2026" dataDxfId="276"/>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0400-00004B000000}" name="Wk 40 2026" dataDxfId="275"/>
-    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0400-00004C000000}" name="Wk 41 2026" dataDxfId="274"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0400-00004D000000}" name="Wk 42 2026" dataDxfId="273"/>
-    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0400-00004E000000}" name="Wk 43 2026" dataDxfId="272"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0400-00004F000000}" name="Wk 44 2026" dataDxfId="271"/>
-    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0400-000050000000}" name="Wk 45 2026" dataDxfId="270"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0400-000051000000}" name="Wk 46 2026" dataDxfId="269"/>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0400-000052000000}" name="Wk 47 2026" dataDxfId="268"/>
-    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0400-000053000000}" name="Wk 48 2026" dataDxfId="267"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0400-000054000000}" name="Wk 49 2026" dataDxfId="266"/>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0400-000055000000}" name="Wk 50 2026" dataDxfId="265"/>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0400-000056000000}" name="Wk 51 2026" dataDxfId="264"/>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0400-000057000000}" name="Wk 52 2026" dataDxfId="263"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0400-00002D000000}" name="Wk 10 2026" dataDxfId="296"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0400-00002E000000}" name="Wk 11 2026" dataDxfId="295"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0400-00002F000000}" name="Wk 12 2026" dataDxfId="294"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0400-000030000000}" name="Wk 13 2026" dataDxfId="293"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0400-000031000000}" name="Wk 14 2026" dataDxfId="292"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0400-000032000000}" name="Wk 15 2026" dataDxfId="291"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0400-000033000000}" name="Wk 16 2026" dataDxfId="290"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0400-000034000000}" name="Wk 17 2026" dataDxfId="289"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0400-000035000000}" name="Wk 18 2026" dataDxfId="288"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0400-000036000000}" name="Wk 19 2026" dataDxfId="287"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0400-000037000000}" name="Wk 20 2026" dataDxfId="286"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0400-000038000000}" name="Wk 21 2026" dataDxfId="285"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0400-000039000000}" name="Wk 22 2026" dataDxfId="284"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0400-00003A000000}" name="Wk 23 2026" dataDxfId="283"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0400-00003B000000}" name="Wk 24 2026" dataDxfId="282"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0400-00003C000000}" name="Wk 25 2026" dataDxfId="281"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0400-00003D000000}" name="Wk 26 2026" dataDxfId="280"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0400-00003E000000}" name="Wk 27 2026" dataDxfId="279"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0400-00003F000000}" name="Wk 28 2026" dataDxfId="278"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0400-000040000000}" name="Wk 29 2026" dataDxfId="277"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0400-000041000000}" name="Wk 30 2026" dataDxfId="276"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0400-000042000000}" name="Wk 31 2026" dataDxfId="275"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0400-000043000000}" name="Wk 32 2026" dataDxfId="274"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0400-000044000000}" name="Wk 33 2026" dataDxfId="273"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0400-000045000000}" name="Wk 34 2026" dataDxfId="272"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0400-000046000000}" name="Wk 35 2026" dataDxfId="271"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0400-000047000000}" name="Wk 36 2026" dataDxfId="270"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0400-000048000000}" name="Wk 37 2026" dataDxfId="269"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0400-000049000000}" name="Wk 38 2026" dataDxfId="268"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0400-00004A000000}" name="Wk 39 2026" dataDxfId="267"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0400-00004B000000}" name="Wk 40 2026" dataDxfId="266"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0400-00004C000000}" name="Wk 41 2026" dataDxfId="265"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0400-00004D000000}" name="Wk 42 2026" dataDxfId="264"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0400-00004E000000}" name="Wk 43 2026" dataDxfId="263"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0400-00004F000000}" name="Wk 44 2026" dataDxfId="262"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0400-000050000000}" name="Wk 45 2026" dataDxfId="261"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0400-000051000000}" name="Wk 46 2026" dataDxfId="260"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0400-000052000000}" name="Wk 47 2026" dataDxfId="259"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0400-000053000000}" name="Wk 48 2026" dataDxfId="258"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0400-000054000000}" name="Wk 49 2026" dataDxfId="257"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0400-000055000000}" name="Wk 50 2026" dataDxfId="256"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0400-000056000000}" name="Wk 51 2026" dataDxfId="255"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0400-000057000000}" name="Wk 52 2026" dataDxfId="254"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblForecastTransits25" displayName="tblForecastTransits25" ref="B14:CJ20" totalsRowShown="0" headerRowDxfId="262" dataDxfId="260" headerRowBorderDxfId="261" tableBorderDxfId="259">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblForecastTransits25" displayName="tblForecastTransits25" ref="B14:CJ20" totalsRowShown="0" headerRowDxfId="253" dataDxfId="251" headerRowBorderDxfId="252" tableBorderDxfId="250">
   <autoFilter ref="B14:CJ20" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="87">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="MP"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Wk19 2025" dataDxfId="258"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Wk20 2025" dataDxfId="257"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Wk21 2025" dataDxfId="256"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Wk22 2025" dataDxfId="255"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wk23 2025" dataDxfId="254"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="Wk24 2025" dataDxfId="253"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Wk25 2025" dataDxfId="252"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="Wk26 2025" dataDxfId="251"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="Wk27 2025" dataDxfId="250"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="Wk28 2025" dataDxfId="249"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="Wk29 2025" dataDxfId="248"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0500-00000D000000}" name="Wk30 2025" dataDxfId="247"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0500-00000E000000}" name="Wk31 2025" dataDxfId="246"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="Wk32 2025" dataDxfId="245"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0500-000010000000}" name="Wk33 2025" dataDxfId="244"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0500-000011000000}" name="Wk34 2025" dataDxfId="243"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0500-000012000000}" name="Wk35 2025" dataDxfId="242"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0500-000013000000}" name="Wk36 2025" dataDxfId="241"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0500-000014000000}" name="Wk37 2025" dataDxfId="240"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0500-000015000000}" name="Wk38 2025" dataDxfId="239"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0500-000016000000}" name="Wk39 2025" dataDxfId="238"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0500-000017000000}" name="Wk40 2025" dataDxfId="237"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0500-000018000000}" name="Wk41 2025" dataDxfId="236"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0500-000019000000}" name="Wk42 2025" dataDxfId="235"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0500-00001A000000}" name="Wk43 2025" dataDxfId="234"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0500-00001B000000}" name="Wk44 2025" dataDxfId="233"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0500-00001C000000}" name="Wk45 2025" dataDxfId="232"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0500-00001D000000}" name="Wk46 2025" dataDxfId="231"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0500-00001E000000}" name="Wk47 2025" dataDxfId="230"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0500-00001F000000}" name="Wk48 2025" dataDxfId="229"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0500-000020000000}" name="Wk49 2025" dataDxfId="228"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0500-000021000000}" name="Wk50 2025" dataDxfId="227"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0500-000022000000}" name="Wk51 2025" dataDxfId="226"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0500-000023000000}" name="Wk52 2025" dataDxfId="225"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0500-000024000000}" name="Wk 1 2026" dataDxfId="224"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0500-000025000000}" name="Wk 2 2026" dataDxfId="223"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0500-000026000000}" name="Wk 3 2026" dataDxfId="222"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0500-000027000000}" name="Wk 4 2026" dataDxfId="221"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0500-000028000000}" name="Wk 5 2026" dataDxfId="220"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0500-000029000000}" name="Wk 6 2026" dataDxfId="219"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0500-00002A000000}" name="Wk 7 2026" dataDxfId="218"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0500-00002B000000}" name="Wk 8 2026" dataDxfId="217"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0500-00002C000000}" name="Wk 9 2026" dataDxfId="216"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0500-00002D000000}" name="Wk 10 2026" dataDxfId="35"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0500-00002E000000}" name="Wk 11 2026" dataDxfId="34"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0500-00002F000000}" name="Wk 12 2026" dataDxfId="33"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0500-000030000000}" name="Wk 13 2026" dataDxfId="32"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0500-000031000000}" name="Wk 14 2026" dataDxfId="31"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0500-000032000000}" name="Wk 15 2026" dataDxfId="30"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0500-000033000000}" name="Wk 16 2026" dataDxfId="29"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0500-000034000000}" name="Wk 17 2026" dataDxfId="28"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0500-000035000000}" name="Wk 18 2026" dataDxfId="27"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0500-000036000000}" name="Wk 19 2026" dataDxfId="215"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0500-000037000000}" name="Wk 20 2026" dataDxfId="214"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0500-000038000000}" name="Wk 21 2026" dataDxfId="213"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0500-000039000000}" name="Wk 22 2026" dataDxfId="212"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0500-00003A000000}" name="Wk 23 2026" dataDxfId="211"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0500-00003B000000}" name="Wk 24 2026" dataDxfId="210"/>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0500-00003C000000}" name="Wk 25 2026" dataDxfId="209"/>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0500-00003D000000}" name="Wk 26 2026" dataDxfId="208"/>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0500-00003E000000}" name="Wk 27 2026" dataDxfId="207"/>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0500-00003F000000}" name="Wk 28 2026" dataDxfId="206"/>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0500-000040000000}" name="Wk 29 2026" dataDxfId="205"/>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0500-000041000000}" name="Wk 30 2026" dataDxfId="204"/>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0500-000042000000}" name="Wk 31 2026" dataDxfId="203"/>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0500-000043000000}" name="Wk 32 2026" dataDxfId="202"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0500-000044000000}" name="Wk 33 2026" dataDxfId="201"/>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0500-000045000000}" name="Wk 34 2026" dataDxfId="200"/>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0500-000046000000}" name="Wk 35 2026" dataDxfId="199"/>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0500-000047000000}" name="Wk 36 2026" dataDxfId="198"/>
-    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0500-000048000000}" name="Wk 37 2026" dataDxfId="197"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0500-000049000000}" name="Wk 38 2026" dataDxfId="196"/>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0500-00004A000000}" name="Wk 39 2026" dataDxfId="195"/>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0500-00004B000000}" name="Wk 40 2026" dataDxfId="194"/>
-    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0500-00004C000000}" name="Wk 41 2026" dataDxfId="193"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0500-00004D000000}" name="Wk 42 2026" dataDxfId="192"/>
-    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0500-00004E000000}" name="Wk 43 2026" dataDxfId="191"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0500-00004F000000}" name="Wk 44 2026" dataDxfId="190"/>
-    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0500-000050000000}" name="Wk 45 2026" dataDxfId="189"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0500-000051000000}" name="Wk 46 2026" dataDxfId="188"/>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0500-000052000000}" name="Wk 47 2026" dataDxfId="187"/>
-    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0500-000053000000}" name="Wk 48 2026" dataDxfId="186"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0500-000054000000}" name="Wk 49 2026" dataDxfId="185"/>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0500-000055000000}" name="Wk 50 2026" dataDxfId="184"/>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0500-000056000000}" name="Wk 51 2026" dataDxfId="183"/>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0500-000057000000}" name="Wk 52 2026" dataDxfId="182"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Wk19 2025" dataDxfId="249"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Wk20 2025" dataDxfId="248"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Wk21 2025" dataDxfId="247"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Wk22 2025" dataDxfId="246"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wk23 2025" dataDxfId="245"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="Wk24 2025" dataDxfId="244"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Wk25 2025" dataDxfId="243"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="Wk26 2025" dataDxfId="242"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="Wk27 2025" dataDxfId="241"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="Wk28 2025" dataDxfId="240"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="Wk29 2025" dataDxfId="239"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0500-00000D000000}" name="Wk30 2025" dataDxfId="238"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0500-00000E000000}" name="Wk31 2025" dataDxfId="237"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="Wk32 2025" dataDxfId="236"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0500-000010000000}" name="Wk33 2025" dataDxfId="235"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0500-000011000000}" name="Wk34 2025" dataDxfId="234"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0500-000012000000}" name="Wk35 2025" dataDxfId="233"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0500-000013000000}" name="Wk36 2025" dataDxfId="232"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0500-000014000000}" name="Wk37 2025" dataDxfId="231"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0500-000015000000}" name="Wk38 2025" dataDxfId="230"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0500-000016000000}" name="Wk39 2025" dataDxfId="229"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0500-000017000000}" name="Wk40 2025" dataDxfId="228"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0500-000018000000}" name="Wk41 2025" dataDxfId="227"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0500-000019000000}" name="Wk42 2025" dataDxfId="226"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0500-00001A000000}" name="Wk43 2025" dataDxfId="225"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0500-00001B000000}" name="Wk44 2025" dataDxfId="224"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0500-00001C000000}" name="Wk45 2025" dataDxfId="223"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0500-00001D000000}" name="Wk46 2025" dataDxfId="222"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0500-00001E000000}" name="Wk47 2025" dataDxfId="221"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0500-00001F000000}" name="Wk48 2025" dataDxfId="220"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0500-000020000000}" name="Wk49 2025" dataDxfId="219"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0500-000021000000}" name="Wk50 2025" dataDxfId="218"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0500-000022000000}" name="Wk51 2025" dataDxfId="217"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0500-000023000000}" name="Wk52 2025" dataDxfId="216"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0500-000024000000}" name="Wk 1 2026" dataDxfId="215"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0500-000025000000}" name="Wk 2 2026" dataDxfId="214"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0500-000026000000}" name="Wk 3 2026" dataDxfId="213"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0500-000027000000}" name="Wk 4 2026" dataDxfId="212"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0500-000028000000}" name="Wk 5 2026" dataDxfId="211"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0500-000029000000}" name="Wk 6 2026" dataDxfId="210"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0500-00002A000000}" name="Wk 7 2026" dataDxfId="209"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0500-00002B000000}" name="Wk 8 2026" dataDxfId="208"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0500-00002C000000}" name="Wk 9 2026" dataDxfId="207"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0500-00002D000000}" name="Wk 10 2026" dataDxfId="206"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0500-00002E000000}" name="Wk 11 2026" dataDxfId="205"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0500-00002F000000}" name="Wk 12 2026" dataDxfId="204"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0500-000030000000}" name="Wk 13 2026" dataDxfId="203"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0500-000031000000}" name="Wk 14 2026" dataDxfId="202"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0500-000032000000}" name="Wk 15 2026" dataDxfId="201"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0500-000033000000}" name="Wk 16 2026" dataDxfId="200"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0500-000034000000}" name="Wk 17 2026" dataDxfId="199"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0500-000035000000}" name="Wk 18 2026" dataDxfId="198"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0500-000036000000}" name="Wk 19 2026" dataDxfId="197"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0500-000037000000}" name="Wk 20 2026" dataDxfId="196"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0500-000038000000}" name="Wk 21 2026" dataDxfId="195"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0500-000039000000}" name="Wk 22 2026" dataDxfId="194"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0500-00003A000000}" name="Wk 23 2026" dataDxfId="193"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0500-00003B000000}" name="Wk 24 2026" dataDxfId="192"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0500-00003C000000}" name="Wk 25 2026" dataDxfId="191"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0500-00003D000000}" name="Wk 26 2026" dataDxfId="190"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0500-00003E000000}" name="Wk 27 2026" dataDxfId="189"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0500-00003F000000}" name="Wk 28 2026" dataDxfId="188"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0500-000040000000}" name="Wk 29 2026" dataDxfId="187"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0500-000041000000}" name="Wk 30 2026" dataDxfId="186"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0500-000042000000}" name="Wk 31 2026" dataDxfId="185"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0500-000043000000}" name="Wk 32 2026" dataDxfId="184"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0500-000044000000}" name="Wk 33 2026" dataDxfId="183"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0500-000045000000}" name="Wk 34 2026" dataDxfId="182"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0500-000046000000}" name="Wk 35 2026" dataDxfId="181"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0500-000047000000}" name="Wk 36 2026" dataDxfId="180"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0500-000048000000}" name="Wk 37 2026" dataDxfId="179"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0500-000049000000}" name="Wk 38 2026" dataDxfId="178"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0500-00004A000000}" name="Wk 39 2026" dataDxfId="177"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0500-00004B000000}" name="Wk 40 2026" dataDxfId="176"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0500-00004C000000}" name="Wk 41 2026" dataDxfId="175"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0500-00004D000000}" name="Wk 42 2026" dataDxfId="174"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0500-00004E000000}" name="Wk 43 2026" dataDxfId="173"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0500-00004F000000}" name="Wk 44 2026" dataDxfId="172"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0500-000050000000}" name="Wk 45 2026" dataDxfId="171"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0500-000051000000}" name="Wk 46 2026" dataDxfId="170"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0500-000052000000}" name="Wk 47 2026" dataDxfId="169"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0500-000053000000}" name="Wk 48 2026" dataDxfId="168"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0500-000054000000}" name="Wk 49 2026" dataDxfId="167"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0500-000055000000}" name="Wk 50 2026" dataDxfId="166"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0500-000056000000}" name="Wk 51 2026" dataDxfId="165"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0500-000057000000}" name="Wk 52 2026" dataDxfId="164"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblForecastConversion26" displayName="tblForecastConversion26" ref="B25:CJ31" totalsRowShown="0" headerRowDxfId="181" headerRowBorderDxfId="180" tableBorderDxfId="179">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tblForecastConversion26" displayName="tblForecastConversion26" ref="B25:CJ31" totalsRowShown="0" headerRowDxfId="163" headerRowBorderDxfId="162" tableBorderDxfId="161">
   <autoFilter ref="B25:CJ31" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <tableColumns count="87">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="MP"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Wk19 2025" dataDxfId="178"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Wk20 2025" dataDxfId="177"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Wk21 2025" dataDxfId="176"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Wk22 2025" dataDxfId="175"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Wk23 2025" dataDxfId="174"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="Wk24 2025" dataDxfId="173"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="Wk25 2025" dataDxfId="172"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="Wk26 2025" dataDxfId="171"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" name="Wk27 2025" dataDxfId="170"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" name="Wk28 2025" dataDxfId="169"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" name="Wk29 2025" dataDxfId="168"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" name="Wk30 2025" dataDxfId="167"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" name="Wk31 2025" dataDxfId="166"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" name="Wk32 2025" dataDxfId="165"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" name="Wk33 2025" dataDxfId="164"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" name="Wk34 2025" dataDxfId="163"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0600-000012000000}" name="Wk35 2025" dataDxfId="162"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0600-000013000000}" name="Wk36 2025" dataDxfId="161"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0600-000014000000}" name="Wk37 2025" dataDxfId="160"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0600-000015000000}" name="Wk38 2025" dataDxfId="159"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0600-000016000000}" name="Wk39 2025" dataDxfId="158"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0600-000017000000}" name="Wk40 2025" dataDxfId="157"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0600-000018000000}" name="Wk41 2025" dataDxfId="156"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0600-000019000000}" name="Wk42 2025" dataDxfId="155"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0600-00001A000000}" name="Wk43 2025" dataDxfId="154"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0600-00001B000000}" name="Wk44 2025" dataDxfId="153"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0600-00001C000000}" name="Wk45 2025" dataDxfId="152"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0600-00001D000000}" name="Wk46 2025" dataDxfId="151"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0600-00001E000000}" name="Wk47 2025" dataDxfId="150"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0600-00001F000000}" name="Wk48 2025" dataDxfId="149"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0600-000020000000}" name="Wk49 2025" dataDxfId="148"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0600-000021000000}" name="Wk50 2025" dataDxfId="147"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0600-000022000000}" name="Wk51 2025" dataDxfId="146"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0600-000023000000}" name="Wk52 2025" dataDxfId="145"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0600-000024000000}" name="Wk 1 2026" dataDxfId="144"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0600-000025000000}" name="Wk 2 2026" dataDxfId="143"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0600-000026000000}" name="Wk 3 2026" dataDxfId="142"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0600-000027000000}" name="Wk 4 2026" dataDxfId="141"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0600-000028000000}" name="Wk 5 2026" dataDxfId="140"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0600-000029000000}" name="Wk 6 2026" dataDxfId="139"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0600-00002A000000}" name="Wk 7 2026" dataDxfId="138"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0600-00002B000000}" name="Wk 8 2026" dataDxfId="137"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0600-00002C000000}" name="Wk 9 2026" dataDxfId="136"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0600-00002D000000}" name="Wk 10 2026" dataDxfId="26"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0600-00002E000000}" name="Wk 11 2026" dataDxfId="25"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0600-00002F000000}" name="Wk 12 2026" dataDxfId="24"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0600-000030000000}" name="Wk 13 2026" dataDxfId="23"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0600-000031000000}" name="Wk 14 2026" dataDxfId="22"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0600-000032000000}" name="Wk 15 2026" dataDxfId="21"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0600-000033000000}" name="Wk 16 2026" dataDxfId="20"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0600-000034000000}" name="Wk 17 2026" dataDxfId="19"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0600-000035000000}" name="Wk 18 2026" dataDxfId="18"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0600-000036000000}" name="Wk 19 2026" dataDxfId="135"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0600-000037000000}" name="Wk 20 2026" dataDxfId="134"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0600-000038000000}" name="Wk 21 2026" dataDxfId="133"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0600-000039000000}" name="Wk 22 2026" dataDxfId="132"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0600-00003A000000}" name="Wk 23 2026" dataDxfId="131"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0600-00003B000000}" name="Wk 24 2026" dataDxfId="130"/>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0600-00003C000000}" name="Wk 25 2026" dataDxfId="129"/>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0600-00003D000000}" name="Wk 26 2026" dataDxfId="128"/>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0600-00003E000000}" name="Wk 27 2026" dataDxfId="127"/>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0600-00003F000000}" name="Wk 28 2026" dataDxfId="126"/>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0600-000040000000}" name="Wk 29 2026" dataDxfId="125"/>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0600-000041000000}" name="Wk 30 2026" dataDxfId="124"/>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0600-000042000000}" name="Wk 31 2026" dataDxfId="123"/>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0600-000043000000}" name="Wk 32 2026" dataDxfId="122"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0600-000044000000}" name="Wk 33 2026" dataDxfId="121"/>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0600-000045000000}" name="Wk 34 2026" dataDxfId="120"/>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0600-000046000000}" name="Wk 35 2026" dataDxfId="119"/>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0600-000047000000}" name="Wk 36 2026" dataDxfId="118"/>
-    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0600-000048000000}" name="Wk 37 2026" dataDxfId="117"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0600-000049000000}" name="Wk 38 2026" dataDxfId="116"/>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0600-00004A000000}" name="Wk 39 2026" dataDxfId="115"/>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0600-00004B000000}" name="Wk 40 2026" dataDxfId="114"/>
-    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0600-00004C000000}" name="Wk 41 2026" dataDxfId="113"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0600-00004D000000}" name="Wk 42 2026" dataDxfId="112"/>
-    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0600-00004E000000}" name="Wk 43 2026" dataDxfId="111"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0600-00004F000000}" name="Wk 44 2026" dataDxfId="110"/>
-    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0600-000050000000}" name="Wk 45 2026" dataDxfId="109"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0600-000051000000}" name="Wk 46 2026" dataDxfId="108"/>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0600-000052000000}" name="Wk 47 2026" dataDxfId="107"/>
-    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0600-000053000000}" name="Wk 48 2026" dataDxfId="106"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0600-000054000000}" name="Wk 49 2026" dataDxfId="105"/>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0600-000055000000}" name="Wk 50 2026" dataDxfId="104"/>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0600-000056000000}" name="Wk 51 2026" dataDxfId="103"/>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0600-000057000000}" name="Wk 52 2026" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Wk19 2025" dataDxfId="160"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Wk20 2025" dataDxfId="159"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Wk21 2025" dataDxfId="158"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Wk22 2025" dataDxfId="157"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Wk23 2025" dataDxfId="156"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="Wk24 2025" dataDxfId="155"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="Wk25 2025" dataDxfId="154"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="Wk26 2025" dataDxfId="153"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" name="Wk27 2025" dataDxfId="152"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" name="Wk28 2025" dataDxfId="151"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" name="Wk29 2025" dataDxfId="150"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" name="Wk30 2025" dataDxfId="149"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" name="Wk31 2025" dataDxfId="148"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" name="Wk32 2025" dataDxfId="147"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" name="Wk33 2025" dataDxfId="146"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" name="Wk34 2025" dataDxfId="145"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0600-000012000000}" name="Wk35 2025" dataDxfId="144"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0600-000013000000}" name="Wk36 2025" dataDxfId="143"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0600-000014000000}" name="Wk37 2025" dataDxfId="142"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0600-000015000000}" name="Wk38 2025" dataDxfId="141"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0600-000016000000}" name="Wk39 2025" dataDxfId="140"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0600-000017000000}" name="Wk40 2025" dataDxfId="139"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0600-000018000000}" name="Wk41 2025" dataDxfId="138"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0600-000019000000}" name="Wk42 2025" dataDxfId="137"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0600-00001A000000}" name="Wk43 2025" dataDxfId="136"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0600-00001B000000}" name="Wk44 2025" dataDxfId="135"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0600-00001C000000}" name="Wk45 2025" dataDxfId="134"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0600-00001D000000}" name="Wk46 2025" dataDxfId="133"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0600-00001E000000}" name="Wk47 2025" dataDxfId="132"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0600-00001F000000}" name="Wk48 2025" dataDxfId="131"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0600-000020000000}" name="Wk49 2025" dataDxfId="130"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0600-000021000000}" name="Wk50 2025" dataDxfId="129"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0600-000022000000}" name="Wk51 2025" dataDxfId="128"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0600-000023000000}" name="Wk52 2025" dataDxfId="127"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0600-000024000000}" name="Wk 1 2026" dataDxfId="126"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0600-000025000000}" name="Wk 2 2026" dataDxfId="125"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0600-000026000000}" name="Wk 3 2026" dataDxfId="124"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0600-000027000000}" name="Wk 4 2026" dataDxfId="123"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0600-000028000000}" name="Wk 5 2026" dataDxfId="122"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0600-000029000000}" name="Wk 6 2026" dataDxfId="121"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0600-00002A000000}" name="Wk 7 2026" dataDxfId="120"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0600-00002B000000}" name="Wk 8 2026" dataDxfId="119"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0600-00002C000000}" name="Wk 9 2026" dataDxfId="118"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0600-00002D000000}" name="Wk 10 2026" dataDxfId="117"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0600-00002E000000}" name="Wk 11 2026" dataDxfId="116"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0600-00002F000000}" name="Wk 12 2026" dataDxfId="115"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0600-000030000000}" name="Wk 13 2026" dataDxfId="114"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0600-000031000000}" name="Wk 14 2026" dataDxfId="113"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0600-000032000000}" name="Wk 15 2026" dataDxfId="112"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0600-000033000000}" name="Wk 16 2026" dataDxfId="111"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0600-000034000000}" name="Wk 17 2026" dataDxfId="110"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0600-000035000000}" name="Wk 18 2026" dataDxfId="109"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0600-000036000000}" name="Wk 19 2026" dataDxfId="108"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0600-000037000000}" name="Wk 20 2026" dataDxfId="107"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0600-000038000000}" name="Wk 21 2026" dataDxfId="106"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0600-000039000000}" name="Wk 22 2026" dataDxfId="105"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0600-00003A000000}" name="Wk 23 2026" dataDxfId="104"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0600-00003B000000}" name="Wk 24 2026" dataDxfId="103"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0600-00003C000000}" name="Wk 25 2026" dataDxfId="102"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0600-00003D000000}" name="Wk 26 2026" dataDxfId="101"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0600-00003E000000}" name="Wk 27 2026" dataDxfId="100"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0600-00003F000000}" name="Wk 28 2026" dataDxfId="99"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0600-000040000000}" name="Wk 29 2026" dataDxfId="98"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0600-000041000000}" name="Wk 30 2026" dataDxfId="97"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0600-000042000000}" name="Wk 31 2026" dataDxfId="96"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0600-000043000000}" name="Wk 32 2026" dataDxfId="95"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0600-000044000000}" name="Wk 33 2026" dataDxfId="94"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0600-000045000000}" name="Wk 34 2026" dataDxfId="93"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0600-000046000000}" name="Wk 35 2026" dataDxfId="92"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0600-000047000000}" name="Wk 36 2026" dataDxfId="91"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0600-000048000000}" name="Wk 37 2026" dataDxfId="90"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0600-000049000000}" name="Wk 38 2026" dataDxfId="89"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0600-00004A000000}" name="Wk 39 2026" dataDxfId="88"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0600-00004B000000}" name="Wk 40 2026" dataDxfId="87"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0600-00004C000000}" name="Wk 41 2026" dataDxfId="86"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0600-00004D000000}" name="Wk 42 2026" dataDxfId="85"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0600-00004E000000}" name="Wk 43 2026" dataDxfId="84"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0600-00004F000000}" name="Wk 44 2026" dataDxfId="83"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0600-000050000000}" name="Wk 45 2026" dataDxfId="82"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0600-000051000000}" name="Wk 46 2026" dataDxfId="81"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0600-000052000000}" name="Wk 47 2026" dataDxfId="80"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0600-000053000000}" name="Wk 48 2026" dataDxfId="79"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0600-000054000000}" name="Wk 49 2026" dataDxfId="78"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0600-000055000000}" name="Wk 50 2026" dataDxfId="77"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0600-000056000000}" name="Wk 51 2026" dataDxfId="76"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0600-000057000000}" name="Wk 52 2026" dataDxfId="75"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="TblForecastUPO27" displayName="TblForecastUPO27" ref="B36:CJ42" totalsRowShown="0" headerRowDxfId="101" headerRowBorderDxfId="100" tableBorderDxfId="99">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="TblForecastUPO27" displayName="TblForecastUPO27" ref="B36:CJ42" totalsRowShown="0" headerRowDxfId="74" headerRowBorderDxfId="73" tableBorderDxfId="72">
   <autoFilter ref="B36:CJ42" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="87">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="MP"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Wk19 2025" dataDxfId="98"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Wk20 2025" dataDxfId="97"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Wk21 2025" dataDxfId="96"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Wk19 2025" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Wk20 2025" dataDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Wk21 2025" dataDxfId="69"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Wk22 2025"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Wk23 2025"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Wk24 2025"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Wk25 2025"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Wk26 2025"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Wk27 2025"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Wk28 2025" dataDxfId="95"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Wk29 2025" dataDxfId="94"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Wk28 2025" dataDxfId="68"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Wk29 2025" dataDxfId="67"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0700-00000D000000}" name="Wk30 2025"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0700-00000E000000}" name="Wk31 2025"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0700-00000F000000}" name="Wk32 2025"/>
@@ -21508,69 +21516,69 @@
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0700-000016000000}" name="Wk39 2025"/>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0700-000017000000}" name="Wk40 2025"/>
     <tableColumn id="24" xr3:uid="{00000000-0010-0000-0700-000018000000}" name="Wk41 2025"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0700-000019000000}" name="Wk42 2025" dataDxfId="93"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0700-00001A000000}" name="Wk43 2025" dataDxfId="92"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0700-00001B000000}" name="Wk44 2025" dataDxfId="91"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0700-00001C000000}" name="Wk45 2025" dataDxfId="90"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="Wk46 2025" dataDxfId="89"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0700-00001E000000}" name="Wk47 2025" dataDxfId="88"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0700-00001F000000}" name="Wk48 2025" dataDxfId="87"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0700-000020000000}" name="Wk49 2025" dataDxfId="86"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0700-000021000000}" name="Wk50 2025" dataDxfId="85"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0700-000022000000}" name="Wk51 2025" dataDxfId="84"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0700-000023000000}" name="Wk52 2025" dataDxfId="83"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0700-000024000000}" name="Wk 1 2026" dataDxfId="82"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0700-000025000000}" name="Wk 2 2026" dataDxfId="81"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0700-000026000000}" name="Wk 3 2026" dataDxfId="80"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0700-000027000000}" name="Wk 4 2026" dataDxfId="79"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0700-000028000000}" name="Wk 5 2026" dataDxfId="78"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0700-000029000000}" name="Wk 6 2026" dataDxfId="77"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0700-00002A000000}" name="Wk 7 2026" dataDxfId="76"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0700-00002B000000}" name="Wk 8 2026" dataDxfId="75"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0700-00002C000000}" name="Wk 9 2026" dataDxfId="74"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0700-00002D000000}" name="Wk 10 2026" dataDxfId="17"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0700-00002E000000}" name="Wk 11 2026" dataDxfId="16"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0700-00002F000000}" name="Wk 12 2026" dataDxfId="15"/>
-    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0700-000030000000}" name="Wk 13 2026" dataDxfId="14"/>
-    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0700-000031000000}" name="Wk 14 2026" dataDxfId="13"/>
-    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0700-000032000000}" name="Wk 15 2026" dataDxfId="12"/>
-    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0700-000033000000}" name="Wk 16 2026" dataDxfId="11"/>
-    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0700-000034000000}" name="Wk 17 2026" dataDxfId="10"/>
-    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0700-000035000000}" name="Wk 18 2026" dataDxfId="9"/>
-    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0700-000036000000}" name="Wk 19 2026" dataDxfId="73"/>
-    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0700-000037000000}" name="Wk 20 2026" dataDxfId="72"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0700-000038000000}" name="Wk 21 2026" dataDxfId="71"/>
-    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0700-000039000000}" name="Wk 22 2026" dataDxfId="70"/>
-    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0700-00003A000000}" name="Wk 23 2026" dataDxfId="69"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0700-00003B000000}" name="Wk 24 2026" dataDxfId="68"/>
-    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0700-00003C000000}" name="Wk 25 2026" dataDxfId="67"/>
-    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0700-00003D000000}" name="Wk 26 2026" dataDxfId="66"/>
-    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0700-00003E000000}" name="Wk 27 2026" dataDxfId="65"/>
-    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0700-00003F000000}" name="Wk 28 2026" dataDxfId="64"/>
-    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0700-000040000000}" name="Wk 29 2026" dataDxfId="63"/>
-    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0700-000041000000}" name="Wk 30 2026" dataDxfId="62"/>
-    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0700-000042000000}" name="Wk 31 2026" dataDxfId="61"/>
-    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0700-000043000000}" name="Wk 32 2026" dataDxfId="60"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0700-000044000000}" name="Wk 33 2026" dataDxfId="59"/>
-    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0700-000045000000}" name="Wk 34 2026" dataDxfId="58"/>
-    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0700-000046000000}" name="Wk 35 2026" dataDxfId="57"/>
-    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0700-000047000000}" name="Wk 36 2026" dataDxfId="56"/>
-    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0700-000048000000}" name="Wk 37 2026" dataDxfId="55"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0700-000049000000}" name="Wk 38 2026" dataDxfId="54"/>
-    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0700-00004A000000}" name="Wk 39 2026" dataDxfId="53"/>
-    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0700-00004B000000}" name="Wk 40 2026" dataDxfId="52"/>
-    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0700-00004C000000}" name="Wk 41 2026" dataDxfId="51"/>
-    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0700-00004D000000}" name="Wk 42 2026" dataDxfId="50"/>
-    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0700-00004E000000}" name="Wk 43 2026" dataDxfId="49"/>
-    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0700-00004F000000}" name="Wk 44 2026" dataDxfId="48"/>
-    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0700-000050000000}" name="Wk 45 2026" dataDxfId="47"/>
-    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0700-000051000000}" name="Wk 46 2026" dataDxfId="46"/>
-    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0700-000052000000}" name="Wk 47 2026" dataDxfId="45"/>
-    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0700-000053000000}" name="Wk 48 2026" dataDxfId="44"/>
-    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0700-000054000000}" name="Wk 49 2026" dataDxfId="43"/>
-    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0700-000055000000}" name="Wk 50 2026" dataDxfId="42"/>
-    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0700-000056000000}" name="Wk 51 2026" dataDxfId="41"/>
-    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0700-000057000000}" name="Wk 52 2026" dataDxfId="40"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0700-000019000000}" name="Wk42 2025" dataDxfId="66"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0700-00001A000000}" name="Wk43 2025" dataDxfId="65"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0700-00001B000000}" name="Wk44 2025" dataDxfId="64"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0700-00001C000000}" name="Wk45 2025" dataDxfId="63"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0700-00001D000000}" name="Wk46 2025" dataDxfId="62"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0700-00001E000000}" name="Wk47 2025" dataDxfId="61"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0700-00001F000000}" name="Wk48 2025" dataDxfId="60"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0700-000020000000}" name="Wk49 2025" dataDxfId="59"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0700-000021000000}" name="Wk50 2025" dataDxfId="58"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0700-000022000000}" name="Wk51 2025" dataDxfId="57"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0700-000023000000}" name="Wk52 2025" dataDxfId="56"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0700-000024000000}" name="Wk 1 2026" dataDxfId="55"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0700-000025000000}" name="Wk 2 2026" dataDxfId="54"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0700-000026000000}" name="Wk 3 2026" dataDxfId="53"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0700-000027000000}" name="Wk 4 2026" dataDxfId="52"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0700-000028000000}" name="Wk 5 2026" dataDxfId="51"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0700-000029000000}" name="Wk 6 2026" dataDxfId="50"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0700-00002A000000}" name="Wk 7 2026" dataDxfId="49"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0700-00002B000000}" name="Wk 8 2026" dataDxfId="48"/>
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0700-00002C000000}" name="Wk 9 2026" dataDxfId="47"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0700-00002D000000}" name="Wk 10 2026" dataDxfId="46"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0700-00002E000000}" name="Wk 11 2026" dataDxfId="45"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0700-00002F000000}" name="Wk 12 2026" dataDxfId="44"/>
+    <tableColumn id="48" xr3:uid="{00000000-0010-0000-0700-000030000000}" name="Wk 13 2026" dataDxfId="43"/>
+    <tableColumn id="49" xr3:uid="{00000000-0010-0000-0700-000031000000}" name="Wk 14 2026" dataDxfId="42"/>
+    <tableColumn id="50" xr3:uid="{00000000-0010-0000-0700-000032000000}" name="Wk 15 2026" dataDxfId="41"/>
+    <tableColumn id="51" xr3:uid="{00000000-0010-0000-0700-000033000000}" name="Wk 16 2026" dataDxfId="40"/>
+    <tableColumn id="52" xr3:uid="{00000000-0010-0000-0700-000034000000}" name="Wk 17 2026" dataDxfId="39"/>
+    <tableColumn id="53" xr3:uid="{00000000-0010-0000-0700-000035000000}" name="Wk 18 2026" dataDxfId="38"/>
+    <tableColumn id="54" xr3:uid="{00000000-0010-0000-0700-000036000000}" name="Wk 19 2026" dataDxfId="37"/>
+    <tableColumn id="55" xr3:uid="{00000000-0010-0000-0700-000037000000}" name="Wk 20 2026" dataDxfId="36"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0700-000038000000}" name="Wk 21 2026" dataDxfId="35"/>
+    <tableColumn id="57" xr3:uid="{00000000-0010-0000-0700-000039000000}" name="Wk 22 2026" dataDxfId="34"/>
+    <tableColumn id="58" xr3:uid="{00000000-0010-0000-0700-00003A000000}" name="Wk 23 2026" dataDxfId="33"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0700-00003B000000}" name="Wk 24 2026" dataDxfId="32"/>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0700-00003C000000}" name="Wk 25 2026" dataDxfId="31"/>
+    <tableColumn id="61" xr3:uid="{00000000-0010-0000-0700-00003D000000}" name="Wk 26 2026" dataDxfId="30"/>
+    <tableColumn id="62" xr3:uid="{00000000-0010-0000-0700-00003E000000}" name="Wk 27 2026" dataDxfId="29"/>
+    <tableColumn id="63" xr3:uid="{00000000-0010-0000-0700-00003F000000}" name="Wk 28 2026" dataDxfId="28"/>
+    <tableColumn id="64" xr3:uid="{00000000-0010-0000-0700-000040000000}" name="Wk 29 2026" dataDxfId="27"/>
+    <tableColumn id="65" xr3:uid="{00000000-0010-0000-0700-000041000000}" name="Wk 30 2026" dataDxfId="26"/>
+    <tableColumn id="66" xr3:uid="{00000000-0010-0000-0700-000042000000}" name="Wk 31 2026" dataDxfId="25"/>
+    <tableColumn id="67" xr3:uid="{00000000-0010-0000-0700-000043000000}" name="Wk 32 2026" dataDxfId="24"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0700-000044000000}" name="Wk 33 2026" dataDxfId="23"/>
+    <tableColumn id="69" xr3:uid="{00000000-0010-0000-0700-000045000000}" name="Wk 34 2026" dataDxfId="22"/>
+    <tableColumn id="70" xr3:uid="{00000000-0010-0000-0700-000046000000}" name="Wk 35 2026" dataDxfId="21"/>
+    <tableColumn id="71" xr3:uid="{00000000-0010-0000-0700-000047000000}" name="Wk 36 2026" dataDxfId="20"/>
+    <tableColumn id="72" xr3:uid="{00000000-0010-0000-0700-000048000000}" name="Wk 37 2026" dataDxfId="19"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0700-000049000000}" name="Wk 38 2026" dataDxfId="18"/>
+    <tableColumn id="74" xr3:uid="{00000000-0010-0000-0700-00004A000000}" name="Wk 39 2026" dataDxfId="17"/>
+    <tableColumn id="75" xr3:uid="{00000000-0010-0000-0700-00004B000000}" name="Wk 40 2026" dataDxfId="16"/>
+    <tableColumn id="76" xr3:uid="{00000000-0010-0000-0700-00004C000000}" name="Wk 41 2026" dataDxfId="15"/>
+    <tableColumn id="77" xr3:uid="{00000000-0010-0000-0700-00004D000000}" name="Wk 42 2026" dataDxfId="14"/>
+    <tableColumn id="78" xr3:uid="{00000000-0010-0000-0700-00004E000000}" name="Wk 43 2026" dataDxfId="13"/>
+    <tableColumn id="79" xr3:uid="{00000000-0010-0000-0700-00004F000000}" name="Wk 44 2026" dataDxfId="12"/>
+    <tableColumn id="80" xr3:uid="{00000000-0010-0000-0700-000050000000}" name="Wk 45 2026" dataDxfId="11"/>
+    <tableColumn id="81" xr3:uid="{00000000-0010-0000-0700-000051000000}" name="Wk 46 2026" dataDxfId="10"/>
+    <tableColumn id="82" xr3:uid="{00000000-0010-0000-0700-000052000000}" name="Wk 47 2026" dataDxfId="9"/>
+    <tableColumn id="83" xr3:uid="{00000000-0010-0000-0700-000053000000}" name="Wk 48 2026" dataDxfId="8"/>
+    <tableColumn id="84" xr3:uid="{00000000-0010-0000-0700-000054000000}" name="Wk 49 2026" dataDxfId="7"/>
+    <tableColumn id="85" xr3:uid="{00000000-0010-0000-0700-000055000000}" name="Wk 50 2026" dataDxfId="6"/>
+    <tableColumn id="86" xr3:uid="{00000000-0010-0000-0700-000056000000}" name="Wk 51 2026" dataDxfId="5"/>
+    <tableColumn id="87" xr3:uid="{00000000-0010-0000-0700-000057000000}" name="Wk 52 2026" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -22301,7 +22309,9 @@
       <c r="AP3" s="1">
         <v>270346</v>
       </c>
-      <c r="AQ3" s="1"/>
+      <c r="AQ3" s="1">
+        <v>246709</v>
+      </c>
       <c r="AR3" s="1"/>
       <c r="AS3" s="1"/>
       <c r="AT3" s="1"/>
@@ -22464,7 +22474,9 @@
       <c r="AP4" s="1">
         <v>67765</v>
       </c>
-      <c r="AQ4" s="1"/>
+      <c r="AQ4" s="1">
+        <v>63217</v>
+      </c>
       <c r="AR4" s="1"/>
       <c r="AS4" s="1"/>
       <c r="AT4" s="1"/>
@@ -22593,7 +22605,9 @@
       <c r="AP5" s="1">
         <v>15525</v>
       </c>
-      <c r="AQ5" s="1"/>
+      <c r="AQ5" s="1">
+        <v>10297</v>
+      </c>
       <c r="AR5" s="1"/>
       <c r="AS5" s="1"/>
       <c r="AT5" s="1"/>
@@ -22722,7 +22736,9 @@
       <c r="AP6" s="1">
         <v>131117</v>
       </c>
-      <c r="AQ6" s="1"/>
+      <c r="AQ6" s="1">
+        <v>123653</v>
+      </c>
       <c r="AR6" s="1"/>
       <c r="AS6" s="1"/>
       <c r="AT6" s="1"/>
@@ -22851,7 +22867,9 @@
       <c r="AP7" s="1">
         <v>89224</v>
       </c>
-      <c r="AQ7" s="1"/>
+      <c r="AQ7" s="1">
+        <v>68216</v>
+      </c>
       <c r="AR7" s="1"/>
       <c r="AS7" s="1"/>
       <c r="AT7" s="1"/>
@@ -23057,7 +23075,9 @@
       <c r="AP8" s="2">
         <v>573977</v>
       </c>
-      <c r="AQ8" s="2"/>
+      <c r="AQ8" s="2">
+        <v>512092</v>
+      </c>
       <c r="AR8" s="2"/>
       <c r="AS8" s="2"/>
       <c r="AT8" s="2"/>
@@ -23496,7 +23516,9 @@
       <c r="AP13" s="2">
         <v>1167002</v>
       </c>
-      <c r="AQ13" s="1"/>
+      <c r="AQ13" s="1">
+        <v>1037609</v>
+      </c>
       <c r="AR13" s="1"/>
       <c r="AS13" s="1"/>
       <c r="AT13" s="1"/>
@@ -23659,7 +23681,9 @@
       <c r="AP14" s="1">
         <v>1565147</v>
       </c>
-      <c r="AQ14" s="1"/>
+      <c r="AQ14" s="1">
+        <v>1214675</v>
+      </c>
       <c r="AR14" s="1"/>
       <c r="AS14" s="1"/>
       <c r="AT14" s="1"/>
@@ -23788,7 +23812,9 @@
       <c r="AP15" s="1">
         <v>427182</v>
       </c>
-      <c r="AQ15" s="1"/>
+      <c r="AQ15" s="1">
+        <v>332528</v>
+      </c>
       <c r="AR15" s="1"/>
       <c r="AS15" s="1"/>
       <c r="AT15" s="1"/>
@@ -23917,7 +23943,9 @@
       <c r="AP16" s="1">
         <v>2010183</v>
       </c>
-      <c r="AQ16" s="1"/>
+      <c r="AQ16" s="1">
+        <v>1896118</v>
+      </c>
       <c r="AR16" s="1"/>
       <c r="AS16" s="1"/>
       <c r="AT16" s="1"/>
@@ -24046,7 +24074,9 @@
       <c r="AP17" s="1">
         <v>1301375</v>
       </c>
-      <c r="AQ17" s="1"/>
+      <c r="AQ17" s="1">
+        <v>1092810</v>
+      </c>
       <c r="AR17" s="1"/>
       <c r="AS17" s="1"/>
       <c r="AT17" s="1"/>
@@ -24253,7 +24283,9 @@
       <c r="AP18" s="2">
         <v>6470889</v>
       </c>
-      <c r="AQ18" s="2"/>
+      <c r="AQ18" s="2">
+        <v>5573740</v>
+      </c>
       <c r="AR18" s="1"/>
       <c r="AS18" s="1"/>
       <c r="AT18" s="1"/>
@@ -24692,7 +24724,9 @@
       <c r="AP22" s="20">
         <v>3.2203886540040208E-2</v>
       </c>
-      <c r="AQ22" s="19"/>
+      <c r="AQ22" s="19">
+        <v>3.4419516407432862E-2</v>
+      </c>
       <c r="AR22" s="19"/>
       <c r="AS22" s="19"/>
       <c r="AT22" s="19"/>
@@ -24855,7 +24889,9 @@
       <c r="AP23" s="19">
         <v>1.102196790461215E-2</v>
       </c>
-      <c r="AQ23" s="19"/>
+      <c r="AQ23" s="19">
+        <v>1.316895465865355E-2</v>
+      </c>
       <c r="AR23" s="19"/>
       <c r="AS23" s="19"/>
       <c r="AT23" s="19"/>
@@ -24984,7 +25020,9 @@
       <c r="AP24" s="19">
         <v>8.3032524778665767E-3</v>
       </c>
-      <c r="AQ24" s="19"/>
+      <c r="AQ24" s="19">
+        <v>7.7286724726940287E-3</v>
+      </c>
       <c r="AR24" s="19"/>
       <c r="AS24" s="19"/>
       <c r="AT24" s="19"/>
@@ -25113,7 +25151,9 @@
       <c r="AP25" s="19">
         <v>8.6882637053442395E-3</v>
       </c>
-      <c r="AQ25" s="19"/>
+      <c r="AQ25" s="19">
+        <v>9.0637818954305595E-3</v>
+      </c>
       <c r="AR25" s="19"/>
       <c r="AS25" s="19"/>
       <c r="AT25" s="19"/>
@@ -25242,7 +25282,9 @@
       <c r="AP26" s="19">
         <v>9.6298146191528197E-3</v>
       </c>
-      <c r="AQ26" s="19"/>
+      <c r="AQ26" s="19">
+        <v>9.1186940090226109E-3</v>
+      </c>
       <c r="AR26" s="19"/>
       <c r="AS26" s="19"/>
       <c r="AT26" s="19"/>
@@ -25449,7 +25491,9 @@
       <c r="AP27" s="20">
         <v>1.365762880494473E-2</v>
       </c>
-      <c r="AQ27" s="20"/>
+      <c r="AQ27" s="20">
+        <v>1.460975933574225E-2</v>
+      </c>
       <c r="AR27" s="19"/>
       <c r="AS27" s="19"/>
       <c r="AT27" s="19"/>
@@ -25889,7 +25933,9 @@
       <c r="AP32" s="32">
         <v>7.1934968868075142</v>
       </c>
-      <c r="AQ32" s="31"/>
+      <c r="AQ32" s="31">
+        <v>6.9079072632581058</v>
+      </c>
       <c r="AR32" s="31"/>
       <c r="AS32" s="31"/>
       <c r="AT32" s="31"/>
@@ -26053,7 +26099,9 @@
       <c r="AP33" s="31">
         <v>3.9281780766332388</v>
       </c>
-      <c r="AQ33" s="31"/>
+      <c r="AQ33" s="31">
+        <v>3.9520505126281571</v>
+      </c>
       <c r="AR33" s="31"/>
       <c r="AS33" s="31"/>
       <c r="AT33" s="31"/>
@@ -26183,7 +26231,9 @@
       <c r="AP34" s="31">
         <v>4.3769382576825491</v>
       </c>
-      <c r="AQ34" s="31"/>
+      <c r="AQ34" s="31">
+        <v>4.0066147859922179</v>
+      </c>
       <c r="AR34" s="31"/>
       <c r="AS34" s="31"/>
       <c r="AT34" s="31"/>
@@ -26313,7 +26363,9 @@
       <c r="AP35" s="31">
         <v>7.5074148296593188</v>
       </c>
-      <c r="AQ35" s="31"/>
+      <c r="AQ35" s="31">
+        <v>7.1949842895379961</v>
+      </c>
       <c r="AR35" s="31"/>
       <c r="AS35" s="31"/>
       <c r="AT35" s="31"/>
@@ -26443,7 +26495,9 @@
       <c r="AP36" s="31">
         <v>7.1196935844238736</v>
       </c>
-      <c r="AQ36" s="31"/>
+      <c r="AQ36" s="31">
+        <v>6.8455594581033621</v>
+      </c>
       <c r="AR36" s="31"/>
       <c r="AS36" s="31"/>
       <c r="AT36" s="31"/>
@@ -26650,7 +26704,9 @@
       <c r="AP37" s="32">
         <v>6.4946422711791527</v>
       </c>
-      <c r="AQ37" s="32"/>
+      <c r="AQ37" s="32">
+        <v>6.2886615662339898</v>
+      </c>
       <c r="AR37" s="31"/>
       <c r="AS37" s="31"/>
       <c r="AT37" s="31"/>
@@ -26730,6 +26786,8 @@
     <col min="38" max="38" width="13.7109375" customWidth="1"/>
     <col min="39" max="41" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="42" max="46" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="47" max="49" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:88" x14ac:dyDescent="0.25">
@@ -27028,7 +27086,7 @@
       <c r="X4" s="37"/>
       <c r="Y4" s="37"/>
       <c r="Z4" s="1">
-        <f t="shared" ref="Z4:BB7" si="0">Z15*Z26*Z37</f>
+        <f t="shared" ref="Z4:AS4" si="0">Z15*Z26*Z37</f>
         <v>69096.999999999782</v>
       </c>
       <c r="AA4" s="1">
@@ -27197,7 +27255,7 @@
       <c r="X5" s="37"/>
       <c r="Y5" s="37"/>
       <c r="Z5" s="1">
-        <f t="shared" ref="Z5:AT5" si="1">Z16*Z27*Z38</f>
+        <f t="shared" ref="Z5:AS5" si="1">Z16*Z27*Z38</f>
         <v>34022.999999999971</v>
       </c>
       <c r="AA5" s="1">
@@ -27366,7 +27424,7 @@
       <c r="X6" s="37"/>
       <c r="Y6" s="37"/>
       <c r="Z6" s="1">
-        <f t="shared" ref="Z6:AT6" si="2">Z17*Z28*Z39</f>
+        <f t="shared" ref="Z6:AS6" si="2">Z17*Z28*Z39</f>
         <v>5299.9999999999882</v>
       </c>
       <c r="AA6" s="1">
@@ -27535,7 +27593,7 @@
       <c r="X7" s="37"/>
       <c r="Y7" s="37"/>
       <c r="Z7" s="1">
-        <f t="shared" ref="Z7:AT7" si="3">Z18*Z29*Z40</f>
+        <f t="shared" ref="Z7:AS7" si="3">Z18*Z29*Z40</f>
         <v>12186.999999999971</v>
       </c>
       <c r="AA7" s="1">
@@ -27704,7 +27762,7 @@
       <c r="X8" s="37"/>
       <c r="Y8" s="37"/>
       <c r="Z8" s="1">
-        <f t="shared" ref="Z8:BB8" si="4">Z19*Z30*Z41</f>
+        <f t="shared" ref="Z8:AS8" si="4">Z19*Z30*Z41</f>
         <v>3516.9999999999741</v>
       </c>
       <c r="AA8" s="1">
@@ -27873,7 +27931,7 @@
       <c r="X9" s="37"/>
       <c r="Y9" s="37"/>
       <c r="Z9" s="1">
-        <f t="shared" ref="Z9:BB9" si="5">SUBTOTAL(109,Z4:Z8)</f>
+        <f t="shared" ref="Z9:AS9" si="5">SUBTOTAL(109,Z4:Z8)</f>
         <v>124123.99999999968</v>
       </c>
       <c r="AA9" s="1">
@@ -29102,7 +29160,7 @@
       <c r="X20" s="36"/>
       <c r="Y20" s="36"/>
       <c r="Z20" s="1">
-        <f t="shared" ref="Z20:AT20" si="6">SUM(Z15:Z19)</f>
+        <f t="shared" ref="Z20:AS20" si="6">SUM(Z15:Z19)</f>
         <v>2683597</v>
       </c>
       <c r="AA20" s="1">
@@ -30284,7 +30342,7 @@
       <c r="X31" s="35"/>
       <c r="Y31" s="35"/>
       <c r="Z31" s="45">
-        <f t="shared" ref="Z31:AT31" si="7">(Z26*Z15+Z16*Z27+Z17*Z28+Z18*Z29+Z19*Z30)/Z20</f>
+        <f t="shared" ref="Z31:AS31" si="7">(Z26*Z15+Z16*Z27+Z17*Z28+Z18*Z29+Z19*Z30)/Z20</f>
         <v>8.4021557633280827E-3</v>
       </c>
       <c r="AA31" s="45">
@@ -31358,7 +31416,7 @@
       <c r="L42" s="34"/>
       <c r="M42" s="34"/>
       <c r="Z42" s="39">
-        <f t="shared" ref="Z42:BB42" si="8">SUM(Z4:Z8)/SUMPRODUCT(Z15:Z19,Z26:Z30)</f>
+        <f t="shared" ref="Z42:AS42" si="8">SUM(Z4:Z8)/SUMPRODUCT(Z15:Z19,Z26:Z30)</f>
         <v>5.5048784814617679</v>
       </c>
       <c r="AA42" s="39">

</xml_diff>